<commit_message>
step9: peak-angle figures as excursion bars + level-walk line, grouped & before ROM
Reworked the named peak-angle figures to read like the ROM figures:
- bars = peak EXCURSION value (begin-ZVP referenced), red dashed line =
  level-walk excursion (gap to the line = change vs level walk; % labels toggle).
  Replaces the earlier Group_PeakDelta_* (zero-line Δ) figures.
- ordered BEFORE the ROM figures.
- grouped anatomically, joint + its IMU segment per figure: hip+thigh,
  knee+shank, ankle+foot; panel titles carry a (P)/(S) role tag.
Paired Δ vs level walk stays in the .md / .xlsx tables (PeakExcursion_deg,
PeakDelta_deg). Includes the matching def_PeakAngles definition figure and the
Step 9 vault note. Regenerated group outputs for 7 participants (101-107).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Results/Group Analysis/GroupCrossing_YoungAdults_Summary.xlsx
+++ b/Results/Group Analysis/GroupCrossing_YoungAdults_Summary.xlsx
@@ -11,6 +11,8 @@
     <sheet name="SegmentROM_deg" sheetId="4" r:id="rId6"/>
     <sheet name="Spatiotemporal" sheetId="5" r:id="rId7"/>
     <sheet name="PeakTiming_pctGC" sheetId="6" r:id="rId8"/>
+    <sheet name="PeakExcursion_deg" sheetId="7" r:id="rId9"/>
+    <sheet name="PeakDelta_deg" sheetId="8" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
@@ -18,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="116" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="190" uniqueCount="79">
   <si>
     <t>Condition</t>
   </si>
@@ -189,6 +191,72 @@
   </si>
   <si>
     <t>Thigh_SD</t>
+  </si>
+  <si>
+    <t>hip_pk_flex_mean</t>
+  </si>
+  <si>
+    <t>hip_pk_flex_SD</t>
+  </si>
+  <si>
+    <t>knee_pk_flex_mean</t>
+  </si>
+  <si>
+    <t>knee_pk_flex_SD</t>
+  </si>
+  <si>
+    <t>ank_dorsi_mean</t>
+  </si>
+  <si>
+    <t>ank_dorsi_SD</t>
+  </si>
+  <si>
+    <t>ank_plant_mean</t>
+  </si>
+  <si>
+    <t>ank_plant_SD</t>
+  </si>
+  <si>
+    <t>hip_pk_ext_mean</t>
+  </si>
+  <si>
+    <t>hip_pk_ext_SD</t>
+  </si>
+  <si>
+    <t>thigh_fwd_mean</t>
+  </si>
+  <si>
+    <t>thigh_fwd_SD</t>
+  </si>
+  <si>
+    <t>shank_back_mean</t>
+  </si>
+  <si>
+    <t>shank_back_SD</t>
+  </si>
+  <si>
+    <t>foot_toedown_mean</t>
+  </si>
+  <si>
+    <t>foot_toedown_SD</t>
+  </si>
+  <si>
+    <t>thigh_back_mean</t>
+  </si>
+  <si>
+    <t>thigh_back_SD</t>
+  </si>
+  <si>
+    <t>shank_fwd_mean</t>
+  </si>
+  <si>
+    <t>shank_fwd_SD</t>
+  </si>
+  <si>
+    <t>foot_toeup_mean</t>
+  </si>
+  <si>
+    <t>foot_toeup_SD</t>
   </si>
 </sst>
 </file>
@@ -294,37 +362,37 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>21.719999999999999</v>
+        <v>21.52</v>
       </c>
       <c r="C2" s="0">
-        <v>4.9199999999999999</v>
+        <v>4.5199999999999996</v>
       </c>
       <c r="D2" s="0">
-        <v>20.27</v>
+        <v>19.359999999999999</v>
       </c>
       <c r="E2" s="0">
-        <v>4.1699999999999999</v>
+        <v>4.5099999999999998</v>
       </c>
       <c r="F2" s="0">
-        <v>18.620000000000001</v>
+        <v>17.66</v>
       </c>
       <c r="G2" s="0">
-        <v>4.5199999999999996</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="H2" s="0">
-        <v>83.239999999999995</v>
+        <v>88.219999999999999</v>
       </c>
       <c r="I2" s="0">
-        <v>16.879999999999999</v>
+        <v>20.280000000000001</v>
       </c>
       <c r="J2" s="0">
-        <v>33.600000000000001</v>
+        <v>32.479999999999997</v>
       </c>
       <c r="K2" s="0">
-        <v>9.8399999999999999</v>
+        <v>9.4600000000000009</v>
       </c>
       <c r="L2" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -332,37 +400,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>17.109999999999999</v>
+        <v>18.02</v>
       </c>
       <c r="C3" s="0">
-        <v>8.3900000000000006</v>
+        <v>8.0299999999999994</v>
       </c>
       <c r="D3" s="0">
-        <v>40.530000000000001</v>
+        <v>39.869999999999997</v>
       </c>
       <c r="E3" s="0">
-        <v>8.1400000000000006</v>
+        <v>7.6299999999999999</v>
       </c>
       <c r="F3" s="0">
-        <v>16.68</v>
+        <v>17.530000000000001</v>
       </c>
       <c r="G3" s="0">
-        <v>8.4800000000000004</v>
+        <v>8.0700000000000003</v>
       </c>
       <c r="H3" s="0">
-        <v>19.079999999999998</v>
+        <v>20.870000000000001</v>
       </c>
       <c r="I3" s="0">
-        <v>5.3700000000000001</v>
+        <v>6.8099999999999996</v>
       </c>
       <c r="J3" s="0">
-        <v>95.900000000000006</v>
+        <v>97.290000000000006</v>
       </c>
       <c r="K3" s="0">
-        <v>14.890000000000001</v>
+        <v>14.08</v>
       </c>
       <c r="L3" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -370,37 +438,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>22.690000000000001</v>
+        <v>22.780000000000001</v>
       </c>
       <c r="C4" s="0">
-        <v>5.4400000000000004</v>
+        <v>4.9699999999999998</v>
       </c>
       <c r="D4" s="0">
-        <v>19.809999999999999</v>
+        <v>18.940000000000001</v>
       </c>
       <c r="E4" s="0">
-        <v>4.4800000000000004</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="F4" s="0">
-        <v>18.640000000000001</v>
+        <v>17.870000000000001</v>
       </c>
       <c r="G4" s="0">
-        <v>4.4800000000000004</v>
+        <v>4.5700000000000003</v>
       </c>
       <c r="H4" s="0">
-        <v>90.200000000000003</v>
+        <v>91.799999999999997</v>
       </c>
       <c r="I4" s="0">
-        <v>16.75</v>
+        <v>15.859999999999999</v>
       </c>
       <c r="J4" s="0">
-        <v>22.98</v>
+        <v>23.949999999999999</v>
       </c>
       <c r="K4" s="0">
-        <v>6.3399999999999999</v>
+        <v>6.3300000000000001</v>
       </c>
       <c r="L4" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -408,37 +476,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>18.25</v>
+        <v>18.550000000000001</v>
       </c>
       <c r="C5" s="0">
-        <v>8.1600000000000001</v>
+        <v>7.4900000000000002</v>
       </c>
       <c r="D5" s="0">
-        <v>41.590000000000003</v>
+        <v>39.539999999999999</v>
       </c>
       <c r="E5" s="0">
-        <v>8.9700000000000006</v>
+        <v>9.8200000000000003</v>
       </c>
       <c r="F5" s="0">
-        <v>17.670000000000002</v>
+        <v>16.850000000000001</v>
       </c>
       <c r="G5" s="0">
-        <v>8.3499999999999996</v>
+        <v>7.9199999999999999</v>
       </c>
       <c r="H5" s="0">
-        <v>26.850000000000001</v>
+        <v>26.300000000000001</v>
       </c>
       <c r="I5" s="0">
-        <v>10.99</v>
+        <v>10.140000000000001</v>
       </c>
       <c r="J5" s="0">
-        <v>91.799999999999997</v>
+        <v>94.280000000000001</v>
       </c>
       <c r="K5" s="0">
-        <v>19.879999999999999</v>
+        <v>19.309999999999999</v>
       </c>
       <c r="L5" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -446,37 +514,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>19.600000000000001</v>
+        <v>18.760000000000002</v>
       </c>
       <c r="C6" s="0">
-        <v>9.3800000000000008</v>
+        <v>8.8399999999999999</v>
       </c>
       <c r="D6" s="0">
-        <v>18.890000000000001</v>
+        <v>17.640000000000001</v>
       </c>
       <c r="E6" s="0">
-        <v>6.1299999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="F6" s="0">
-        <v>16.539999999999999</v>
+        <v>15.359999999999999</v>
       </c>
       <c r="G6" s="0">
-        <v>7.7199999999999998</v>
+        <v>7.71</v>
       </c>
       <c r="H6" s="0">
-        <v>83.959999999999994</v>
+        <v>88.299999999999997</v>
       </c>
       <c r="I6" s="0">
-        <v>22.559999999999999</v>
+        <v>23.59</v>
       </c>
       <c r="J6" s="0">
-        <v>24.440000000000001</v>
+        <v>24.140000000000001</v>
       </c>
       <c r="K6" s="0">
-        <v>7.4500000000000002</v>
+        <v>6.8399999999999999</v>
       </c>
       <c r="L6" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -484,37 +552,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>15.75</v>
+        <v>15.449999999999999</v>
       </c>
       <c r="C7" s="0">
-        <v>7.4400000000000004</v>
+        <v>6.8300000000000001</v>
       </c>
       <c r="D7" s="0">
-        <v>36.439999999999998</v>
+        <v>34.579999999999998</v>
       </c>
       <c r="E7" s="0">
-        <v>3.7400000000000002</v>
+        <v>5.9800000000000004</v>
       </c>
       <c r="F7" s="0">
-        <v>15.27</v>
+        <v>14.43</v>
       </c>
       <c r="G7" s="0">
-        <v>7.29</v>
+        <v>7.0099999999999998</v>
       </c>
       <c r="H7" s="0">
-        <v>19.059999999999999</v>
+        <v>20.02</v>
       </c>
       <c r="I7" s="0">
-        <v>6.3799999999999999</v>
+        <v>6.3399999999999999</v>
       </c>
       <c r="J7" s="0">
-        <v>90.620000000000005</v>
+        <v>92.439999999999998</v>
       </c>
       <c r="K7" s="0">
-        <v>26.460000000000001</v>
+        <v>24.620000000000001</v>
       </c>
       <c r="L7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -522,37 +590,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>22.690000000000001</v>
+        <v>24</v>
       </c>
       <c r="C8" s="0">
-        <v>6.2400000000000002</v>
+        <v>6.6699999999999999</v>
       </c>
       <c r="D8" s="0">
-        <v>19.440000000000001</v>
+        <v>20.109999999999999</v>
       </c>
       <c r="E8" s="0">
-        <v>5.8399999999999999</v>
+        <v>5.6200000000000001</v>
       </c>
       <c r="F8" s="0">
-        <v>16.710000000000001</v>
+        <v>17.010000000000002</v>
       </c>
       <c r="G8" s="0">
-        <v>5.6100000000000003</v>
+        <v>5.1799999999999997</v>
       </c>
       <c r="H8" s="0">
-        <v>90.200000000000003</v>
+        <v>90.409999999999997</v>
       </c>
       <c r="I8" s="0">
-        <v>21.899999999999999</v>
+        <v>20</v>
       </c>
       <c r="J8" s="0">
-        <v>22.359999999999999</v>
+        <v>26.289999999999999</v>
       </c>
       <c r="K8" s="0">
-        <v>13.17</v>
+        <v>15.890000000000001</v>
       </c>
       <c r="L8" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -560,37 +628,37 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>20.010000000000002</v>
+        <v>21.239999999999998</v>
       </c>
       <c r="C9" s="0">
-        <v>5.2800000000000002</v>
+        <v>5.8099999999999996</v>
       </c>
       <c r="D9" s="0">
-        <v>42.759999999999998</v>
+        <v>40.659999999999997</v>
       </c>
       <c r="E9" s="0">
-        <v>6.0599999999999996</v>
+        <v>7.8499999999999996</v>
       </c>
       <c r="F9" s="0">
-        <v>17.609999999999999</v>
+        <v>17.809999999999999</v>
       </c>
       <c r="G9" s="0">
-        <v>5.9699999999999998</v>
+        <v>5.4800000000000004</v>
       </c>
       <c r="H9" s="0">
-        <v>20.789999999999999</v>
+        <v>19.969999999999999</v>
       </c>
       <c r="I9" s="0">
-        <v>8.6300000000000008</v>
+        <v>8.1699999999999999</v>
       </c>
       <c r="J9" s="0">
-        <v>90.010000000000005</v>
+        <v>92.239999999999995</v>
       </c>
       <c r="K9" s="0">
-        <v>17.41</v>
+        <v>16.949999999999999</v>
       </c>
       <c r="L9" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -598,37 +666,37 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>23.600000000000001</v>
+        <v>23.210000000000001</v>
       </c>
       <c r="C10" s="0">
-        <v>6.4199999999999999</v>
+        <v>5.9500000000000002</v>
       </c>
       <c r="D10" s="0">
-        <v>22.170000000000002</v>
+        <v>22.010000000000002</v>
       </c>
       <c r="E10" s="0">
-        <v>5.0300000000000002</v>
+        <v>4.6100000000000003</v>
       </c>
       <c r="F10" s="0">
-        <v>18.129999999999999</v>
+        <v>17.710000000000001</v>
       </c>
       <c r="G10" s="0">
-        <v>5.6200000000000001</v>
+        <v>5.25</v>
       </c>
       <c r="H10" s="0">
-        <v>85.040000000000006</v>
+        <v>87.75</v>
       </c>
       <c r="I10" s="0">
-        <v>19.129999999999999</v>
+        <v>18.879999999999999</v>
       </c>
       <c r="J10" s="0">
-        <v>19.149999999999999</v>
+        <v>19.390000000000001</v>
       </c>
       <c r="K10" s="0">
-        <v>6.5899999999999999</v>
+        <v>6.0499999999999998</v>
       </c>
       <c r="L10" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -636,37 +704,37 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>18.600000000000001</v>
+        <v>20.899999999999999</v>
       </c>
       <c r="C11" s="0">
-        <v>8.4299999999999997</v>
+        <v>9.8200000000000003</v>
       </c>
       <c r="D11" s="0">
-        <v>41.460000000000001</v>
+        <v>41.149999999999999</v>
       </c>
       <c r="E11" s="0">
-        <v>8.0500000000000007</v>
+        <v>7.3899999999999997</v>
       </c>
       <c r="F11" s="0">
-        <v>15.76</v>
+        <v>17.789999999999999</v>
       </c>
       <c r="G11" s="0">
-        <v>9.3000000000000007</v>
+        <v>10.050000000000001</v>
       </c>
       <c r="H11" s="0">
-        <v>17.809999999999999</v>
+        <v>18.620000000000001</v>
       </c>
       <c r="I11" s="0">
-        <v>5.75</v>
+        <v>5.6699999999999999</v>
       </c>
       <c r="J11" s="0">
-        <v>80.299999999999997</v>
+        <v>83.349999999999994</v>
       </c>
       <c r="K11" s="0">
-        <v>25.07</v>
+        <v>24.27</v>
       </c>
       <c r="L11" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -674,37 +742,37 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>21.199999999999999</v>
+        <v>21.82</v>
       </c>
       <c r="C12" s="0">
-        <v>6.3300000000000001</v>
+        <v>6</v>
       </c>
       <c r="D12" s="0">
-        <v>20.399999999999999</v>
+        <v>20.68</v>
       </c>
       <c r="E12" s="0">
-        <v>4.46</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="F12" s="0">
-        <v>16.530000000000001</v>
+        <v>16.82</v>
       </c>
       <c r="G12" s="0">
-        <v>4.7300000000000004</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="H12" s="0">
-        <v>85.859999999999999</v>
+        <v>87.489999999999995</v>
       </c>
       <c r="I12" s="0">
-        <v>21.120000000000001</v>
+        <v>19.75</v>
       </c>
       <c r="J12" s="0">
-        <v>21.73</v>
+        <v>20.75</v>
       </c>
       <c r="K12" s="0">
-        <v>14.859999999999999</v>
+        <v>13.81</v>
       </c>
       <c r="L12" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -712,37 +780,37 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>20.719999999999999</v>
+        <v>22.609999999999999</v>
       </c>
       <c r="C13" s="0">
-        <v>8.6300000000000008</v>
+        <v>9.3200000000000003</v>
       </c>
       <c r="D13" s="0">
-        <v>41.880000000000003</v>
+        <v>43.189999999999998</v>
       </c>
       <c r="E13" s="0">
-        <v>8.8599999999999994</v>
+        <v>8.8100000000000005</v>
       </c>
       <c r="F13" s="0">
-        <v>17.739999999999998</v>
+        <v>19.16</v>
       </c>
       <c r="G13" s="0">
-        <v>7.7800000000000002</v>
+        <v>8.0399999999999991</v>
       </c>
       <c r="H13" s="0">
-        <v>18.25</v>
+        <v>18.460000000000001</v>
       </c>
       <c r="I13" s="0">
-        <v>7.1900000000000004</v>
+        <v>6.5899999999999999</v>
       </c>
       <c r="J13" s="0">
-        <v>88.329999999999998</v>
+        <v>89.109999999999999</v>
       </c>
       <c r="K13" s="0">
-        <v>17.760000000000002</v>
+        <v>16.34</v>
       </c>
       <c r="L13" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -795,25 +863,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>72.599999999999994</v>
+        <v>67.700000000000003</v>
       </c>
       <c r="C2" s="0">
-        <v>53.700000000000003</v>
+        <v>23</v>
       </c>
       <c r="D2" s="0">
-        <v>96.5</v>
+        <v>84.799999999999997</v>
       </c>
       <c r="E2" s="0">
-        <v>92.700000000000003</v>
+        <v>32</v>
       </c>
       <c r="F2" s="0">
-        <v>60.799999999999997</v>
+        <v>61.799999999999997</v>
       </c>
       <c r="G2" s="0">
-        <v>38.200000000000003</v>
+        <v>28</v>
       </c>
       <c r="H2" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -821,25 +889,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>45.700000000000003</v>
+        <v>44</v>
       </c>
       <c r="C3" s="0">
-        <v>9.4000000000000004</v>
+        <v>16</v>
       </c>
       <c r="D3" s="0">
-        <v>72.5</v>
+        <v>72.099999999999994</v>
       </c>
       <c r="E3" s="0">
-        <v>31.5</v>
+        <v>28.199999999999999</v>
       </c>
       <c r="F3" s="0">
-        <v>95.299999999999997</v>
+        <v>94.5</v>
       </c>
       <c r="G3" s="0">
-        <v>61.799999999999997</v>
+        <v>31</v>
       </c>
       <c r="H3" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -847,25 +915,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>80.599999999999994</v>
+        <v>76.400000000000006</v>
       </c>
       <c r="C4" s="0">
-        <v>48.5</v>
+        <v>28</v>
       </c>
       <c r="D4" s="0">
-        <v>100</v>
+        <v>90.200000000000003</v>
       </c>
       <c r="E4" s="0">
-        <v>87.200000000000003</v>
+        <v>37</v>
       </c>
       <c r="F4" s="0">
-        <v>54.200000000000003</v>
+        <v>55.100000000000001</v>
       </c>
       <c r="G4" s="0">
-        <v>37</v>
+        <v>33.899999999999999</v>
       </c>
       <c r="H4" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -873,25 +941,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>51.299999999999997</v>
+        <v>50.5</v>
       </c>
       <c r="C5" s="0">
-        <v>14.199999999999999</v>
+        <v>13.1</v>
       </c>
       <c r="D5" s="0">
-        <v>70.200000000000003</v>
+        <v>74.900000000000006</v>
       </c>
       <c r="E5" s="0">
-        <v>32.899999999999999</v>
+        <v>32.5</v>
       </c>
       <c r="F5" s="0">
-        <v>96.900000000000006</v>
+        <v>98.599999999999994</v>
       </c>
       <c r="G5" s="0">
-        <v>64.599999999999994</v>
+        <v>29</v>
       </c>
       <c r="H5" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -899,25 +967,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>85.5</v>
+        <v>83.5</v>
       </c>
       <c r="C6" s="0">
-        <v>50.600000000000001</v>
+        <v>30</v>
       </c>
       <c r="D6" s="0">
-        <v>105.5</v>
+        <v>96.200000000000003</v>
       </c>
       <c r="E6" s="0">
-        <v>82.200000000000003</v>
+        <v>28</v>
       </c>
       <c r="F6" s="0">
-        <v>55.399999999999999</v>
+        <v>56.899999999999999</v>
       </c>
       <c r="G6" s="0">
-        <v>29.600000000000001</v>
+        <v>27.300000000000001</v>
       </c>
       <c r="H6" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -925,25 +993,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>62.299999999999997</v>
+        <v>60.899999999999999</v>
       </c>
       <c r="C7" s="0">
-        <v>18</v>
+        <v>16.5</v>
       </c>
       <c r="D7" s="0">
-        <v>85.200000000000003</v>
+        <v>86.400000000000006</v>
       </c>
       <c r="E7" s="0">
-        <v>20.100000000000001</v>
+        <v>18.199999999999999</v>
       </c>
       <c r="F7" s="0">
-        <v>121.40000000000001</v>
+        <v>118.2</v>
       </c>
       <c r="G7" s="0">
-        <v>50.100000000000001</v>
+        <v>28</v>
       </c>
       <c r="H7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -951,25 +1019,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>68</v>
+        <v>65.400000000000006</v>
       </c>
       <c r="C8" s="0">
-        <v>51.600000000000001</v>
+        <v>21</v>
       </c>
       <c r="D8" s="0">
-        <v>88.700000000000003</v>
+        <v>81.200000000000003</v>
       </c>
       <c r="E8" s="0">
-        <v>83.5</v>
+        <v>27</v>
       </c>
       <c r="F8" s="0">
-        <v>62.799999999999997</v>
+        <v>63.200000000000003</v>
       </c>
       <c r="G8" s="0">
-        <v>39.100000000000001</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="H8" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -977,25 +1045,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>42.700000000000003</v>
+        <v>42.899999999999999</v>
       </c>
       <c r="C9" s="0">
-        <v>9.4000000000000004</v>
+        <v>8.5999999999999996</v>
       </c>
       <c r="D9" s="0">
-        <v>76.400000000000006</v>
+        <v>77.700000000000003</v>
       </c>
       <c r="E9" s="0">
-        <v>25.5</v>
+        <v>23.600000000000001</v>
       </c>
       <c r="F9" s="0">
-        <v>89.599999999999994</v>
+        <v>91.5</v>
       </c>
       <c r="G9" s="0">
-        <v>58.200000000000003</v>
+        <v>27</v>
       </c>
       <c r="H9" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1003,25 +1071,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>83.299999999999997</v>
+        <v>80.5</v>
       </c>
       <c r="C10" s="0">
-        <v>44.299999999999997</v>
+        <v>14</v>
       </c>
       <c r="D10" s="0">
-        <v>102.59999999999999</v>
+        <v>94.400000000000006</v>
       </c>
       <c r="E10" s="0">
-        <v>69.5</v>
+        <v>26</v>
       </c>
       <c r="F10" s="0">
-        <v>55.600000000000001</v>
+        <v>55.700000000000003</v>
       </c>
       <c r="G10" s="0">
-        <v>34.399999999999999</v>
+        <v>31.399999999999999</v>
       </c>
       <c r="H10" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1029,25 +1097,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>51.700000000000003</v>
+        <v>52.899999999999999</v>
       </c>
       <c r="C11" s="0">
-        <v>16.100000000000001</v>
+        <v>15</v>
       </c>
       <c r="D11" s="0">
-        <v>68.599999999999994</v>
+        <v>71.200000000000003</v>
       </c>
       <c r="E11" s="0">
-        <v>26.199999999999999</v>
+        <v>24.899999999999999</v>
       </c>
       <c r="F11" s="0">
-        <v>96.700000000000003</v>
+        <v>96.599999999999994</v>
       </c>
       <c r="G11" s="0">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="H11" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1055,25 +1123,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>86.599999999999994</v>
+        <v>84.900000000000006</v>
       </c>
       <c r="C12" s="0">
-        <v>53.899999999999999</v>
+        <v>23</v>
       </c>
       <c r="D12" s="0">
-        <v>109.59999999999999</v>
+        <v>100.90000000000001</v>
       </c>
       <c r="E12" s="0">
-        <v>84.799999999999997</v>
+        <v>31</v>
       </c>
       <c r="F12" s="0">
-        <v>65.799999999999997</v>
+        <v>65.700000000000003</v>
       </c>
       <c r="G12" s="0">
-        <v>32.299999999999997</v>
+        <v>29.5</v>
       </c>
       <c r="H12" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1081,25 +1149,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>68.599999999999994</v>
+        <v>69.700000000000003</v>
       </c>
       <c r="C13" s="0">
-        <v>19.5</v>
+        <v>17.699999999999999</v>
       </c>
       <c r="D13" s="0">
-        <v>92.400000000000006</v>
+        <v>89.900000000000006</v>
       </c>
       <c r="E13" s="0">
-        <v>29.899999999999999</v>
+        <v>27.399999999999999</v>
       </c>
       <c r="F13" s="0">
-        <v>103.2</v>
+        <v>100.90000000000001</v>
       </c>
       <c r="G13" s="0">
-        <v>60.200000000000003</v>
+        <v>29</v>
       </c>
       <c r="H13" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1107,25 +1175,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="0">
-        <v>24.5</v>
+        <v>24.300000000000001</v>
       </c>
       <c r="C14" s="0">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="D14" s="0">
-        <v>38.200000000000003</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="E14" s="0">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="F14" s="0">
-        <v>51</v>
+        <v>54.100000000000001</v>
       </c>
       <c r="G14" s="0">
-        <v>26</v>
+        <v>25.199999999999999</v>
       </c>
       <c r="H14" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1178,25 +1246,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>93.400000000000006</v>
+        <v>94.799999999999997</v>
       </c>
       <c r="C2" s="0">
-        <v>13.699999999999999</v>
+        <v>13</v>
       </c>
       <c r="D2" s="0">
-        <v>79.299999999999997</v>
+        <v>80.200000000000003</v>
       </c>
       <c r="E2" s="0">
-        <v>7.2999999999999998</v>
+        <v>7</v>
       </c>
       <c r="F2" s="0">
-        <v>84.200000000000003</v>
+        <v>83.700000000000003</v>
       </c>
       <c r="G2" s="0">
-        <v>11</v>
+        <v>9.9000000000000004</v>
       </c>
       <c r="H2" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1204,25 +1272,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>114.59999999999999</v>
+        <v>112.40000000000001</v>
       </c>
       <c r="C3" s="0">
-        <v>20.399999999999999</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="D3" s="0">
-        <v>106.2</v>
+        <v>104.90000000000001</v>
       </c>
       <c r="E3" s="0">
-        <v>16.100000000000001</v>
+        <v>15.1</v>
       </c>
       <c r="F3" s="0">
-        <v>60.799999999999997</v>
+        <v>60.399999999999999</v>
       </c>
       <c r="G3" s="0">
-        <v>6.4000000000000004</v>
+        <v>5.7999999999999998</v>
       </c>
       <c r="H3" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1230,25 +1298,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>90.799999999999997</v>
+        <v>91.5</v>
       </c>
       <c r="C4" s="0">
-        <v>19.5</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="D4" s="0">
-        <v>82.299999999999997</v>
+        <v>82.400000000000006</v>
       </c>
       <c r="E4" s="0">
-        <v>8</v>
+        <v>7.2999999999999998</v>
       </c>
       <c r="F4" s="0">
-        <v>96.5</v>
+        <v>96.099999999999994</v>
       </c>
       <c r="G4" s="0">
-        <v>9.0999999999999996</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="H4" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -1256,25 +1324,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>120.40000000000001</v>
+        <v>119</v>
       </c>
       <c r="C5" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="0">
-        <v>117</v>
+        <v>116.59999999999999</v>
       </c>
       <c r="E5" s="0">
-        <v>13.6</v>
+        <v>12.4</v>
       </c>
       <c r="F5" s="0">
-        <v>62</v>
+        <v>61.799999999999997</v>
       </c>
       <c r="G5" s="0">
-        <v>5.7999999999999998</v>
+        <v>5.2999999999999998</v>
       </c>
       <c r="H5" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -1282,25 +1350,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>84.5</v>
+        <v>85.799999999999997</v>
       </c>
       <c r="C6" s="0">
-        <v>17.600000000000001</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="D6" s="0">
-        <v>83</v>
+        <v>83.099999999999994</v>
       </c>
       <c r="E6" s="0">
-        <v>6.0999999999999996</v>
+        <v>5.5999999999999996</v>
       </c>
       <c r="F6" s="0">
-        <v>103.2</v>
+        <v>103.90000000000001</v>
       </c>
       <c r="G6" s="0">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="H6" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1308,25 +1376,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>124.40000000000001</v>
+        <v>122</v>
       </c>
       <c r="C7" s="0">
-        <v>21.199999999999999</v>
+        <v>20.300000000000001</v>
       </c>
       <c r="D7" s="0">
-        <v>124.7</v>
+        <v>123.3</v>
       </c>
       <c r="E7" s="0">
-        <v>6.7999999999999998</v>
+        <v>7.2999999999999998</v>
       </c>
       <c r="F7" s="0">
         <v>65.599999999999994</v>
       </c>
       <c r="G7" s="0">
-        <v>7.7000000000000002</v>
+        <v>6.7999999999999998</v>
       </c>
       <c r="H7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1334,25 +1402,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>98.700000000000003</v>
+        <v>99.299999999999997</v>
       </c>
       <c r="C8" s="0">
-        <v>19.399999999999999</v>
+        <v>17.800000000000001</v>
       </c>
       <c r="D8" s="0">
-        <v>82.200000000000003</v>
+        <v>83</v>
       </c>
       <c r="E8" s="0">
-        <v>7.2000000000000002</v>
+        <v>6.9000000000000004</v>
       </c>
       <c r="F8" s="0">
-        <v>84</v>
+        <v>84.400000000000006</v>
       </c>
       <c r="G8" s="0">
-        <v>10.699999999999999</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="H8" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1360,25 +1428,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>119.7</v>
+        <v>117.59999999999999</v>
       </c>
       <c r="C9" s="0">
-        <v>19.399999999999999</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="D9" s="0">
-        <v>106.90000000000001</v>
+        <v>106.7</v>
       </c>
       <c r="E9" s="0">
-        <v>14.6</v>
+        <v>13.300000000000001</v>
       </c>
       <c r="F9" s="0">
-        <v>61.600000000000001</v>
+        <v>61.399999999999999</v>
       </c>
       <c r="G9" s="0">
-        <v>7.4000000000000004</v>
+        <v>6.7999999999999998</v>
       </c>
       <c r="H9" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1386,25 +1454,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C10" s="0">
-        <v>21.199999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="D10" s="0">
-        <v>84.700000000000003</v>
+        <v>84.900000000000006</v>
       </c>
       <c r="E10" s="0">
-        <v>7.0999999999999996</v>
+        <v>6.5</v>
       </c>
       <c r="F10" s="0">
-        <v>97.200000000000003</v>
+        <v>97.700000000000003</v>
       </c>
       <c r="G10" s="0">
-        <v>8.4000000000000004</v>
+        <v>7.7999999999999998</v>
       </c>
       <c r="H10" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1412,25 +1480,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>119.2</v>
+        <v>117.8</v>
       </c>
       <c r="C11" s="0">
-        <v>17.899999999999999</v>
+        <v>16.800000000000001</v>
       </c>
       <c r="D11" s="0">
-        <v>116.3</v>
+        <v>115.8</v>
       </c>
       <c r="E11" s="0">
-        <v>11.5</v>
+        <v>10.6</v>
       </c>
       <c r="F11" s="0">
-        <v>62.600000000000001</v>
+        <v>63.200000000000003</v>
       </c>
       <c r="G11" s="0">
-        <v>7.2000000000000002</v>
+        <v>6.7999999999999998</v>
       </c>
       <c r="H11" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1438,25 +1506,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>87.599999999999994</v>
+        <v>86.099999999999994</v>
       </c>
       <c r="C12" s="0">
-        <v>17.699999999999999</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="D12" s="0">
-        <v>82.299999999999997</v>
+        <v>82.599999999999994</v>
       </c>
       <c r="E12" s="0">
-        <v>5.2999999999999998</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="F12" s="0">
-        <v>107.09999999999999</v>
+        <v>106.90000000000001</v>
       </c>
       <c r="G12" s="0">
-        <v>10.199999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="H12" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1464,25 +1532,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>129.59999999999999</v>
+        <v>126.90000000000001</v>
       </c>
       <c r="C13" s="0">
         <v>17.5</v>
       </c>
       <c r="D13" s="0">
-        <v>133.80000000000001</v>
+        <v>132.40000000000001</v>
       </c>
       <c r="E13" s="0">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="F13" s="0">
-        <v>68.099999999999994</v>
+        <v>67.900000000000006</v>
       </c>
       <c r="G13" s="0">
-        <v>10.800000000000001</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="H13" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1490,25 +1558,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="0">
-        <v>92.5</v>
+        <v>92.400000000000006</v>
       </c>
       <c r="C14" s="0">
-        <v>8.5</v>
+        <v>7.7999999999999998</v>
       </c>
       <c r="D14" s="0">
-        <v>74.900000000000006</v>
+        <v>75.200000000000003</v>
       </c>
       <c r="E14" s="0">
-        <v>5.9000000000000004</v>
+        <v>5.5</v>
       </c>
       <c r="F14" s="0">
-        <v>45.299999999999997</v>
+        <v>45.200000000000003</v>
       </c>
       <c r="G14" s="0">
-        <v>4.9000000000000004</v>
+        <v>4.5</v>
       </c>
       <c r="H14" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1561,25 +1629,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>160.28999999999999</v>
+        <v>163.46000000000001</v>
       </c>
       <c r="C2" s="0">
-        <v>16.52</v>
+        <v>17.25</v>
       </c>
       <c r="D2" s="0">
-        <v>87.150000000000006</v>
+        <v>86.489999999999995</v>
       </c>
       <c r="E2" s="0">
-        <v>9.5</v>
+        <v>8.8499999999999996</v>
       </c>
       <c r="F2" s="0">
-        <v>1.1100000000000001</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="G2" s="0">
         <v>0.17000000000000001</v>
       </c>
       <c r="H2" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1587,25 +1655,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>156.61000000000001</v>
+        <v>159.18000000000001</v>
       </c>
       <c r="C3" s="0">
-        <v>23.469999999999999</v>
+        <v>22.469999999999999</v>
       </c>
       <c r="D3" s="0">
-        <v>81.650000000000006</v>
+        <v>82.299999999999997</v>
       </c>
       <c r="E3" s="0">
-        <v>5.04</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="F3" s="0">
-        <v>1.05</v>
+        <v>1.0800000000000001</v>
       </c>
       <c r="G3" s="0">
         <v>0.17000000000000001</v>
       </c>
       <c r="H3" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1613,25 +1681,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>162.41999999999999</v>
+        <v>163.49000000000001</v>
       </c>
       <c r="C4" s="0">
-        <v>34.509999999999998</v>
+        <v>31.629999999999999</v>
       </c>
       <c r="D4" s="0">
-        <v>83.75</v>
+        <v>82.989999999999995</v>
       </c>
       <c r="E4" s="0">
-        <v>6.4299999999999997</v>
+        <v>6.2000000000000002</v>
       </c>
       <c r="F4" s="0">
         <v>1.0900000000000001</v>
       </c>
       <c r="G4" s="0">
-        <v>0.17000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="H4" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -1639,25 +1707,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>156.16</v>
+        <v>158.33000000000001</v>
       </c>
       <c r="C5" s="0">
-        <v>28.690000000000001</v>
+        <v>26.809999999999999</v>
       </c>
       <c r="D5" s="0">
-        <v>77.349999999999994</v>
+        <v>77.650000000000006</v>
       </c>
       <c r="E5" s="0">
-        <v>4.5999999999999996</v>
+        <v>4.2800000000000002</v>
       </c>
       <c r="F5" s="0">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="G5" s="0">
-        <v>0.22</v>
+        <v>0.20999999999999999</v>
       </c>
       <c r="H5" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -1665,25 +1733,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>151.97999999999999</v>
+        <v>155.71000000000001</v>
       </c>
       <c r="C6" s="0">
-        <v>30</v>
+        <v>29.120000000000001</v>
       </c>
       <c r="D6" s="0">
-        <v>79.060000000000002</v>
+        <v>78.219999999999999</v>
       </c>
       <c r="E6" s="0">
-        <v>6.5700000000000003</v>
+        <v>6.4000000000000004</v>
       </c>
       <c r="F6" s="0">
-        <v>0.97999999999999998</v>
+        <v>1</v>
       </c>
       <c r="G6" s="0">
-        <v>0.22</v>
+        <v>0.20999999999999999</v>
       </c>
       <c r="H6" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1691,25 +1759,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>155.87</v>
+        <v>157.71000000000001</v>
       </c>
       <c r="C7" s="0">
-        <v>39.369999999999997</v>
+        <v>36.270000000000003</v>
       </c>
       <c r="D7" s="0">
-        <v>73.310000000000002</v>
+        <v>73.739999999999995</v>
       </c>
       <c r="E7" s="0">
-        <v>5</v>
+        <v>4.71</v>
       </c>
       <c r="F7" s="0">
-        <v>0.93999999999999995</v>
+        <v>0.95999999999999996</v>
       </c>
       <c r="G7" s="0">
-        <v>0.25</v>
+        <v>0.23000000000000001</v>
       </c>
       <c r="H7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1717,25 +1785,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>161.22</v>
+        <v>164.16999999999999</v>
       </c>
       <c r="C8" s="0">
-        <v>23.739999999999998</v>
+        <v>23.030000000000001</v>
       </c>
       <c r="D8" s="0">
-        <v>87.370000000000005</v>
+        <v>86.450000000000003</v>
       </c>
       <c r="E8" s="0">
-        <v>9.0299999999999994</v>
+        <v>8.5999999999999996</v>
       </c>
       <c r="F8" s="0">
-        <v>1.1399999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="G8" s="0">
-        <v>0.20999999999999999</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="H8" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1743,25 +1811,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>158.37</v>
+        <v>160.66999999999999</v>
       </c>
       <c r="C9" s="0">
-        <v>24.460000000000001</v>
+        <v>23.140000000000001</v>
       </c>
       <c r="D9" s="0">
-        <v>83.540000000000006</v>
+        <v>83.799999999999997</v>
       </c>
       <c r="E9" s="0">
-        <v>5.9100000000000001</v>
+        <v>5.4400000000000004</v>
       </c>
       <c r="F9" s="0">
-        <v>1.1100000000000001</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="G9" s="0">
-        <v>0.20999999999999999</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="H9" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1769,25 +1837,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>150.00999999999999</v>
+        <v>153.50999999999999</v>
       </c>
       <c r="C10" s="0">
-        <v>26.219999999999999</v>
+        <v>25.649999999999999</v>
       </c>
       <c r="D10" s="0">
-        <v>81.480000000000004</v>
+        <v>80.709999999999994</v>
       </c>
       <c r="E10" s="0">
-        <v>4.3099999999999996</v>
+        <v>4.4400000000000004</v>
       </c>
       <c r="F10" s="0">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="G10" s="0">
-        <v>0.22</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="H10" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1795,25 +1863,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>144.18000000000001</v>
+        <v>148.66999999999999</v>
       </c>
       <c r="C11" s="0">
-        <v>32.770000000000003</v>
+        <v>32.18</v>
       </c>
       <c r="D11" s="0">
-        <v>80.900000000000006</v>
+        <v>80.439999999999998</v>
       </c>
       <c r="E11" s="0">
-        <v>10.16</v>
+        <v>9.3499999999999996</v>
       </c>
       <c r="F11" s="0">
-        <v>0.93999999999999995</v>
+        <v>0.96999999999999997</v>
       </c>
       <c r="G11" s="0">
-        <v>0.22</v>
+        <v>0.20999999999999999</v>
       </c>
       <c r="H11" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1821,25 +1889,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>147.05000000000001</v>
+        <v>149.49000000000001</v>
       </c>
       <c r="C12" s="0">
-        <v>38.859999999999999</v>
+        <v>36.049999999999997</v>
       </c>
       <c r="D12" s="0">
-        <v>86.200000000000003</v>
+        <v>84.099999999999994</v>
       </c>
       <c r="E12" s="0">
-        <v>17.670000000000002</v>
+        <v>17.059999999999999</v>
       </c>
       <c r="F12" s="0">
         <v>0.95999999999999996</v>
       </c>
       <c r="G12" s="0">
-        <v>0.20999999999999999</v>
+        <v>0.19</v>
       </c>
       <c r="H12" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1847,25 +1915,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>156.94999999999999</v>
+        <v>157.96000000000001</v>
       </c>
       <c r="C13" s="0">
-        <v>28</v>
+        <v>25.699999999999999</v>
       </c>
       <c r="D13" s="0">
-        <v>71.030000000000001</v>
+        <v>70.700000000000003</v>
       </c>
       <c r="E13" s="0">
-        <v>7.2800000000000002</v>
+        <v>6.7000000000000002</v>
       </c>
       <c r="F13" s="0">
-        <v>0.91000000000000003</v>
+        <v>0.92000000000000004</v>
       </c>
       <c r="G13" s="0">
-        <v>0.19</v>
+        <v>0.17000000000000001</v>
       </c>
       <c r="H13" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1873,25 +1941,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="0">
-        <v>127.84999999999999</v>
+        <v>131.63</v>
       </c>
       <c r="C14" s="0">
-        <v>16.469999999999999</v>
+        <v>18.050000000000001</v>
       </c>
       <c r="D14" s="0">
-        <v>96.549999999999997</v>
+        <v>96.290000000000006</v>
       </c>
       <c r="E14" s="0">
-        <v>4.0899999999999999</v>
+        <v>3.7999999999999998</v>
       </c>
       <c r="F14" s="0">
-        <v>1.03</v>
+        <v>1.0600000000000001</v>
       </c>
       <c r="G14" s="0">
         <v>0.17000000000000001</v>
       </c>
       <c r="H14" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1976,49 +2044,49 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>38.420000000000002</v>
+        <v>40.640000000000001</v>
       </c>
       <c r="C2" s="0">
-        <v>23.640000000000001</v>
+        <v>21.829999999999998</v>
       </c>
       <c r="D2" s="0">
-        <v>52.609999999999999</v>
+        <v>51.079999999999998</v>
       </c>
       <c r="E2" s="0">
-        <v>12.460000000000001</v>
+        <v>11.76</v>
       </c>
       <c r="F2" s="0">
-        <v>44.689999999999998</v>
+        <v>48.049999999999997</v>
       </c>
       <c r="G2" s="0">
-        <v>9.0700000000000003</v>
+        <v>12.16</v>
       </c>
       <c r="H2" s="0">
-        <v>49.299999999999997</v>
+        <v>49.280000000000001</v>
       </c>
       <c r="I2" s="0">
-        <v>4.2999999999999998</v>
+        <v>3.9199999999999999</v>
       </c>
       <c r="J2" s="0">
-        <v>35.409999999999997</v>
+        <v>34.75</v>
       </c>
       <c r="K2" s="0">
-        <v>4.6799999999999997</v>
+        <v>4.6200000000000001</v>
       </c>
       <c r="L2" s="0">
-        <v>36.32</v>
+        <v>35.859999999999999</v>
       </c>
       <c r="M2" s="0">
-        <v>3.5099999999999998</v>
+        <v>3.4300000000000002</v>
       </c>
       <c r="N2" s="0">
-        <v>51.100000000000001</v>
+        <v>51.479999999999997</v>
       </c>
       <c r="O2" s="0">
-        <v>5.4900000000000002</v>
+        <v>5</v>
       </c>
       <c r="P2" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -2026,49 +2094,49 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>34.039999999999999</v>
+        <v>37.329999999999998</v>
       </c>
       <c r="C3" s="0">
-        <v>36.240000000000002</v>
+        <v>33.399999999999999</v>
       </c>
       <c r="D3" s="0">
-        <v>58.420000000000002</v>
+        <v>56.82</v>
       </c>
       <c r="E3" s="0">
-        <v>3.8500000000000001</v>
+        <v>5.21</v>
       </c>
       <c r="F3" s="0">
-        <v>60.439999999999998</v>
+        <v>58.490000000000002</v>
       </c>
       <c r="G3" s="0">
-        <v>16.800000000000001</v>
+        <v>16.18</v>
       </c>
       <c r="H3" s="0">
-        <v>52.350000000000001</v>
+        <v>51.859999999999999</v>
       </c>
       <c r="I3" s="0">
-        <v>6.2800000000000002</v>
+        <v>5.8799999999999999</v>
       </c>
       <c r="J3" s="0">
-        <v>47.840000000000003</v>
+        <v>46.729999999999997</v>
       </c>
       <c r="K3" s="0">
-        <v>5.8300000000000001</v>
+        <v>6.0700000000000003</v>
       </c>
       <c r="L3" s="0">
-        <v>48.909999999999997</v>
+        <v>48.43</v>
       </c>
       <c r="M3" s="0">
-        <v>5.4100000000000001</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="N3" s="0">
-        <v>61.600000000000001</v>
+        <v>60.979999999999997</v>
       </c>
       <c r="O3" s="0">
-        <v>6.6799999999999997</v>
+        <v>6.1600000000000001</v>
       </c>
       <c r="P3" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -2076,49 +2144,49 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>40.799999999999997</v>
+        <v>41.909999999999997</v>
       </c>
       <c r="C4" s="0">
-        <v>20.050000000000001</v>
+        <v>18.539999999999999</v>
       </c>
       <c r="D4" s="0">
-        <v>52.060000000000002</v>
+        <v>50.280000000000001</v>
       </c>
       <c r="E4" s="0">
-        <v>24.579999999999998</v>
+        <v>22.920000000000002</v>
       </c>
       <c r="F4" s="0">
-        <v>46.850000000000001</v>
+        <v>49.630000000000003</v>
       </c>
       <c r="G4" s="0">
-        <v>17.030000000000001</v>
+        <v>17.199999999999999</v>
       </c>
       <c r="H4" s="0">
-        <v>50.600000000000001</v>
+        <v>50.060000000000002</v>
       </c>
       <c r="I4" s="0">
-        <v>7.3200000000000003</v>
+        <v>6.8399999999999999</v>
       </c>
       <c r="J4" s="0">
-        <v>33.32</v>
+        <v>32.509999999999998</v>
       </c>
       <c r="K4" s="0">
-        <v>6.1200000000000001</v>
+        <v>5.9900000000000002</v>
       </c>
       <c r="L4" s="0">
-        <v>36.229999999999997</v>
+        <v>35.530000000000001</v>
       </c>
       <c r="M4" s="0">
-        <v>6.7000000000000002</v>
+        <v>6.3899999999999997</v>
       </c>
       <c r="N4" s="0">
-        <v>51.189999999999998</v>
+        <v>50.979999999999997</v>
       </c>
       <c r="O4" s="0">
-        <v>7.4900000000000002</v>
+        <v>6.8600000000000003</v>
       </c>
       <c r="P4" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -2126,49 +2194,49 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>33.18</v>
+        <v>36.310000000000002</v>
       </c>
       <c r="C5" s="0">
-        <v>29.170000000000002</v>
+        <v>27.879999999999999</v>
       </c>
       <c r="D5" s="0">
-        <v>59.359999999999999</v>
+        <v>58.049999999999997</v>
       </c>
       <c r="E5" s="0">
-        <v>7</v>
+        <v>7.2599999999999998</v>
       </c>
       <c r="F5" s="0">
-        <v>52.310000000000002</v>
+        <v>51.990000000000002</v>
       </c>
       <c r="G5" s="0">
-        <v>23.449999999999999</v>
+        <v>21.43</v>
       </c>
       <c r="H5" s="0">
-        <v>55.780000000000001</v>
+        <v>55.020000000000003</v>
       </c>
       <c r="I5" s="0">
-        <v>0.98999999999999999</v>
+        <v>2.21</v>
       </c>
       <c r="J5" s="0">
-        <v>51.390000000000001</v>
+        <v>50.619999999999997</v>
       </c>
       <c r="K5" s="0">
-        <v>1.02</v>
+        <v>2.23</v>
       </c>
       <c r="L5" s="0">
-        <v>52.659999999999997</v>
+        <v>52.020000000000003</v>
       </c>
       <c r="M5" s="0">
-        <v>1.53</v>
+        <v>2.21</v>
       </c>
       <c r="N5" s="0">
-        <v>64.659999999999997</v>
+        <v>63.909999999999997</v>
       </c>
       <c r="O5" s="0">
-        <v>2</v>
+        <v>2.7000000000000002</v>
       </c>
       <c r="P5" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -2176,49 +2244,49 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>31.600000000000001</v>
+        <v>34.509999999999998</v>
       </c>
       <c r="C6" s="0">
-        <v>26.010000000000002</v>
+        <v>24.329999999999998</v>
       </c>
       <c r="D6" s="0">
-        <v>49.530000000000001</v>
+        <v>48.020000000000003</v>
       </c>
       <c r="E6" s="0">
-        <v>13.92</v>
+        <v>12.98</v>
       </c>
       <c r="F6" s="0">
-        <v>36.68</v>
+        <v>40.259999999999998</v>
       </c>
       <c r="G6" s="0">
-        <v>19.559999999999999</v>
+        <v>20.210000000000001</v>
       </c>
       <c r="H6" s="0">
-        <v>47.390000000000001</v>
+        <v>47.68</v>
       </c>
       <c r="I6" s="0">
-        <v>5.5300000000000002</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="J6" s="0">
-        <v>28.809999999999999</v>
+        <v>28.640000000000001</v>
       </c>
       <c r="K6" s="0">
-        <v>4.8399999999999999</v>
+        <v>4.4400000000000004</v>
       </c>
       <c r="L6" s="0">
-        <v>32.799999999999997</v>
+        <v>32.219999999999999</v>
       </c>
       <c r="M6" s="0">
-        <v>6.4000000000000004</v>
+        <v>6.04</v>
       </c>
       <c r="N6" s="0">
-        <v>47.020000000000003</v>
+        <v>47.710000000000001</v>
       </c>
       <c r="O6" s="0">
-        <v>6.6900000000000004</v>
+        <v>6.2199999999999998</v>
       </c>
       <c r="P6" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -2226,49 +2294,49 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>30.75</v>
+        <v>36.109999999999999</v>
       </c>
       <c r="C7" s="0">
-        <v>29.460000000000001</v>
+        <v>29.440000000000001</v>
       </c>
       <c r="D7" s="0">
-        <v>60.780000000000001</v>
+        <v>59.359999999999999</v>
       </c>
       <c r="E7" s="0">
-        <v>8.0500000000000007</v>
+        <v>7.9900000000000002</v>
       </c>
       <c r="F7" s="0">
-        <v>60.939999999999998</v>
+        <v>60.390000000000001</v>
       </c>
       <c r="G7" s="0">
-        <v>16.949999999999999</v>
+        <v>15.539999999999999</v>
       </c>
       <c r="H7" s="0">
-        <v>54.340000000000003</v>
+        <v>54.130000000000003</v>
       </c>
       <c r="I7" s="0">
-        <v>3.1099999999999999</v>
+        <v>2.8900000000000001</v>
       </c>
       <c r="J7" s="0">
-        <v>51.420000000000002</v>
+        <v>51.07</v>
       </c>
       <c r="K7" s="0">
-        <v>2.8799999999999999</v>
+        <v>2.79</v>
       </c>
       <c r="L7" s="0">
-        <v>51.609999999999999</v>
+        <v>51.469999999999999</v>
       </c>
       <c r="M7" s="0">
-        <v>2.8799999999999999</v>
+        <v>2.6600000000000001</v>
       </c>
       <c r="N7" s="0">
-        <v>64.719999999999999</v>
+        <v>64.090000000000003</v>
       </c>
       <c r="O7" s="0">
-        <v>2.96</v>
+        <v>3.0800000000000001</v>
       </c>
       <c r="P7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -2276,49 +2344,49 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>35.700000000000003</v>
+        <v>37.829999999999998</v>
       </c>
       <c r="C8" s="0">
-        <v>16.890000000000001</v>
+        <v>16.420000000000002</v>
       </c>
       <c r="D8" s="0">
-        <v>42.659999999999997</v>
+        <v>42.18</v>
       </c>
       <c r="E8" s="0">
-        <v>19.100000000000001</v>
+        <v>17.48</v>
       </c>
       <c r="F8" s="0">
-        <v>50.57</v>
+        <v>52.810000000000002</v>
       </c>
       <c r="G8" s="0">
-        <v>15.52</v>
+        <v>15.359999999999999</v>
       </c>
       <c r="H8" s="0">
-        <v>47.920000000000002</v>
+        <v>47.75</v>
       </c>
       <c r="I8" s="0">
-        <v>6.3099999999999996</v>
+        <v>5.7800000000000002</v>
       </c>
       <c r="J8" s="0">
-        <v>34.560000000000002</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="K8" s="0">
-        <v>3.8700000000000001</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="L8" s="0">
-        <v>36.920000000000002</v>
+        <v>36.119999999999997</v>
       </c>
       <c r="M8" s="0">
-        <v>4.4299999999999997</v>
+        <v>4.5499999999999998</v>
       </c>
       <c r="N8" s="0">
-        <v>52.520000000000003</v>
+        <v>52.310000000000002</v>
       </c>
       <c r="O8" s="0">
-        <v>5.7400000000000002</v>
+        <v>5.2699999999999996</v>
       </c>
       <c r="P8" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -2326,49 +2394,49 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>28.390000000000001</v>
+        <v>33.090000000000003</v>
       </c>
       <c r="C9" s="0">
-        <v>15.58</v>
+        <v>18.890000000000001</v>
       </c>
       <c r="D9" s="0">
-        <v>59.170000000000002</v>
+        <v>57.719999999999999</v>
       </c>
       <c r="E9" s="0">
-        <v>9.7799999999999994</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="F9" s="0">
-        <v>57.090000000000003</v>
+        <v>55.810000000000002</v>
       </c>
       <c r="G9" s="0">
-        <v>14.73</v>
+        <v>13.869999999999999</v>
       </c>
       <c r="H9" s="0">
-        <v>54.560000000000002</v>
+        <v>53.840000000000003</v>
       </c>
       <c r="I9" s="0">
-        <v>1.55</v>
+        <v>2.3599999999999999</v>
       </c>
       <c r="J9" s="0">
-        <v>49.18</v>
+        <v>48.460000000000001</v>
       </c>
       <c r="K9" s="0">
-        <v>3.1200000000000001</v>
+        <v>3.4300000000000002</v>
       </c>
       <c r="L9" s="0">
-        <v>51.210000000000001</v>
+        <v>50.579999999999998</v>
       </c>
       <c r="M9" s="0">
-        <v>2.48</v>
+        <v>2.7999999999999998</v>
       </c>
       <c r="N9" s="0">
-        <v>63.990000000000002</v>
+        <v>63.18</v>
       </c>
       <c r="O9" s="0">
-        <v>2.8399999999999999</v>
+        <v>3.3700000000000001</v>
       </c>
       <c r="P9" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -2376,49 +2444,49 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>34.200000000000003</v>
+        <v>36.799999999999997</v>
       </c>
       <c r="C10" s="0">
-        <v>21.030000000000001</v>
+        <v>20.390000000000001</v>
       </c>
       <c r="D10" s="0">
-        <v>52.969999999999999</v>
+        <v>50.880000000000003</v>
       </c>
       <c r="E10" s="0">
-        <v>23.07</v>
+        <v>21.780000000000001</v>
       </c>
       <c r="F10" s="0">
-        <v>39.5</v>
+        <v>42.579999999999998</v>
       </c>
       <c r="G10" s="0">
-        <v>15.68</v>
+        <v>16.48</v>
       </c>
       <c r="H10" s="0">
-        <v>50.670000000000002</v>
+        <v>50.219999999999999</v>
       </c>
       <c r="I10" s="0">
-        <v>3.6600000000000001</v>
+        <v>3.5499999999999998</v>
       </c>
       <c r="J10" s="0">
-        <v>29.649999999999999</v>
+        <v>29.260000000000002</v>
       </c>
       <c r="K10" s="0">
-        <v>3.9900000000000002</v>
+        <v>3.7799999999999998</v>
       </c>
       <c r="L10" s="0">
-        <v>33.18</v>
+        <v>32.880000000000003</v>
       </c>
       <c r="M10" s="0">
-        <v>4.3700000000000001</v>
+        <v>4.0700000000000003</v>
       </c>
       <c r="N10" s="0">
-        <v>51.609999999999999</v>
+        <v>51.399999999999999</v>
       </c>
       <c r="O10" s="0">
-        <v>4.0999999999999996</v>
+        <v>3.7799999999999998</v>
       </c>
       <c r="P10" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -2426,49 +2494,49 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>29.449999999999999</v>
+        <v>33.640000000000001</v>
       </c>
       <c r="C11" s="0">
-        <v>23.59</v>
+        <v>24.23</v>
       </c>
       <c r="D11" s="0">
-        <v>51.259999999999998</v>
+        <v>51.159999999999997</v>
       </c>
       <c r="E11" s="0">
-        <v>9.3399999999999999</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="F11" s="0">
-        <v>58.189999999999998</v>
+        <v>57.799999999999997</v>
       </c>
       <c r="G11" s="0">
-        <v>17.190000000000001</v>
+        <v>15.73</v>
       </c>
       <c r="H11" s="0">
-        <v>55.630000000000003</v>
+        <v>54.990000000000002</v>
       </c>
       <c r="I11" s="0">
-        <v>1.1699999999999999</v>
+        <v>2</v>
       </c>
       <c r="J11" s="0">
-        <v>53.700000000000003</v>
+        <v>52.659999999999997</v>
       </c>
       <c r="K11" s="0">
-        <v>5.5999999999999996</v>
+        <v>5.8099999999999996</v>
       </c>
       <c r="L11" s="0">
-        <v>54.859999999999999</v>
+        <v>53.899999999999999</v>
       </c>
       <c r="M11" s="0">
-        <v>5.7599999999999998</v>
+        <v>5.8399999999999999</v>
       </c>
       <c r="N11" s="0">
-        <v>66.549999999999997</v>
+        <v>65.560000000000002</v>
       </c>
       <c r="O11" s="0">
-        <v>5.6100000000000003</v>
+        <v>5.75</v>
       </c>
       <c r="P11" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -2476,49 +2544,49 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>49.670000000000002</v>
+        <v>49.899999999999999</v>
       </c>
       <c r="C12" s="0">
-        <v>17.620000000000001</v>
+        <v>15.77</v>
       </c>
       <c r="D12" s="0">
-        <v>48.159999999999997</v>
+        <v>46.869999999999997</v>
       </c>
       <c r="E12" s="0">
-        <v>21.07</v>
+        <v>19.109999999999999</v>
       </c>
       <c r="F12" s="0">
-        <v>44.560000000000002</v>
+        <v>43.799999999999997</v>
       </c>
       <c r="G12" s="0">
-        <v>10.43</v>
+        <v>9.7400000000000002</v>
       </c>
       <c r="H12" s="0">
-        <v>52.039999999999999</v>
+        <v>51.490000000000002</v>
       </c>
       <c r="I12" s="0">
-        <v>8.4499999999999993</v>
+        <v>7.8499999999999996</v>
       </c>
       <c r="J12" s="0">
-        <v>34.509999999999998</v>
+        <v>33.43</v>
       </c>
       <c r="K12" s="0">
-        <v>5.6299999999999999</v>
+        <v>5.8799999999999999</v>
       </c>
       <c r="L12" s="0">
-        <v>38.280000000000001</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="M12" s="0">
-        <v>5.6699999999999999</v>
+        <v>5.7800000000000002</v>
       </c>
       <c r="N12" s="0">
-        <v>56.109999999999999</v>
+        <v>55.100000000000001</v>
       </c>
       <c r="O12" s="0">
-        <v>11.67</v>
+        <v>10.720000000000001</v>
       </c>
       <c r="P12" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -2526,49 +2594,49 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>31.960000000000001</v>
+        <v>38.390000000000001</v>
       </c>
       <c r="C13" s="0">
-        <v>28.920000000000002</v>
+        <v>30.289999999999999</v>
       </c>
       <c r="D13" s="0">
-        <v>62.960000000000001</v>
+        <v>61.280000000000001</v>
       </c>
       <c r="E13" s="0">
-        <v>9.5500000000000007</v>
+        <v>9.4800000000000004</v>
       </c>
       <c r="F13" s="0">
-        <v>56.299999999999997</v>
+        <v>57.189999999999998</v>
       </c>
       <c r="G13" s="0">
-        <v>21.800000000000001</v>
+        <v>20.039999999999999</v>
       </c>
       <c r="H13" s="0">
-        <v>54.990000000000002</v>
+        <v>54.700000000000003</v>
       </c>
       <c r="I13" s="0">
-        <v>3.5899999999999999</v>
+        <v>3.3700000000000001</v>
       </c>
       <c r="J13" s="0">
-        <v>51.659999999999997</v>
+        <v>51.479999999999997</v>
       </c>
       <c r="K13" s="0">
-        <v>2.98</v>
+        <v>2.77</v>
       </c>
       <c r="L13" s="0">
-        <v>52.380000000000003</v>
+        <v>52.130000000000003</v>
       </c>
       <c r="M13" s="0">
-        <v>3</v>
+        <v>2.8199999999999998</v>
       </c>
       <c r="N13" s="0">
-        <v>65.719999999999999</v>
+        <v>65.109999999999999</v>
       </c>
       <c r="O13" s="0">
-        <v>3.8700000000000001</v>
+        <v>3.7599999999999998</v>
       </c>
       <c r="P13" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -2576,49 +2644,2191 @@
         <v>24</v>
       </c>
       <c r="B14" s="0">
-        <v>43.140000000000001</v>
+        <v>45.119999999999997</v>
       </c>
       <c r="C14" s="0">
-        <v>19.98</v>
+        <v>18.98</v>
       </c>
       <c r="D14" s="0">
-        <v>53.810000000000002</v>
+        <v>52.990000000000002</v>
       </c>
       <c r="E14" s="0">
-        <v>10.27</v>
+        <v>9.6199999999999992</v>
       </c>
       <c r="F14" s="0">
-        <v>46.380000000000003</v>
+        <v>47.109999999999999</v>
       </c>
       <c r="G14" s="0">
-        <v>5.79</v>
+        <v>5.6299999999999999</v>
       </c>
       <c r="H14" s="0">
-        <v>56.579999999999998</v>
+        <v>55.859999999999999</v>
       </c>
       <c r="I14" s="0">
-        <v>10.279999999999999</v>
+        <v>9.5800000000000001</v>
       </c>
       <c r="J14" s="0">
-        <v>39.259999999999998</v>
+        <v>38.710000000000001</v>
       </c>
       <c r="K14" s="0">
-        <v>1.28</v>
+        <v>1.8600000000000001</v>
       </c>
       <c r="L14" s="0">
-        <v>40.18</v>
+        <v>39.619999999999997</v>
       </c>
       <c r="M14" s="0">
-        <v>2.2799999999999998</v>
+        <v>2.5600000000000001</v>
       </c>
       <c r="N14" s="0">
-        <v>67.530000000000001</v>
+        <v>67.939999999999998</v>
       </c>
       <c r="O14" s="0">
-        <v>7.9199999999999999</v>
+        <v>7.3099999999999996</v>
       </c>
       <c r="P14" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" customWidth="true"/>
+    <col min="2" max="2" width="17.5703125" customWidth="true"/>
+    <col min="3" max="3" width="14.85546875" customWidth="true"/>
+    <col min="4" max="4" width="19.140625" customWidth="true"/>
+    <col min="5" max="5" width="16.42578125" customWidth="true"/>
+    <col min="6" max="6" width="15.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13" customWidth="true"/>
+    <col min="8" max="8" width="15.85546875" customWidth="true"/>
+    <col min="9" max="9" width="13.140625" customWidth="true"/>
+    <col min="10" max="10" width="17" customWidth="true"/>
+    <col min="11" max="11" width="14.28515625" customWidth="true"/>
+    <col min="12" max="12" width="16.140625" customWidth="true"/>
+    <col min="13" max="13" width="13.42578125" customWidth="true"/>
+    <col min="14" max="14" width="17.28515625" customWidth="true"/>
+    <col min="15" max="15" width="14.5703125" customWidth="true"/>
+    <col min="16" max="16" width="19.85546875" customWidth="true"/>
+    <col min="17" max="17" width="17.140625" customWidth="true"/>
+    <col min="18" max="18" width="16.7109375" customWidth="true"/>
+    <col min="19" max="19" width="14" customWidth="true"/>
+    <col min="20" max="20" width="16.7109375" customWidth="true"/>
+    <col min="21" max="21" width="14" customWidth="true"/>
+    <col min="22" max="22" width="17.140625" customWidth="true"/>
+    <col min="23" max="23" width="14.42578125" customWidth="true"/>
+    <col min="24" max="24" width="13.7109375" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="T1" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>45.530000000000001</v>
+      </c>
+      <c r="C2" s="0">
+        <v>51.189999999999998</v>
+      </c>
+      <c r="D2" s="0">
+        <v>52.960000000000001</v>
+      </c>
+      <c r="E2" s="0">
+        <v>84.890000000000001</v>
+      </c>
+      <c r="F2" s="0">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="G2" s="0">
+        <v>25.870000000000001</v>
+      </c>
+      <c r="H2" s="0">
+        <v>28.140000000000001</v>
+      </c>
+      <c r="I2" s="0">
+        <v>16.809999999999999</v>
+      </c>
+      <c r="J2" s="0">
+        <v>22.16</v>
+      </c>
+      <c r="K2" s="0">
+        <v>8.25</v>
+      </c>
+      <c r="L2" s="0">
+        <v>62.880000000000003</v>
+      </c>
+      <c r="M2" s="0">
+        <v>12.16</v>
+      </c>
+      <c r="N2" s="0">
+        <v>52.009999999999998</v>
+      </c>
+      <c r="O2" s="0">
+        <v>6.5800000000000001</v>
+      </c>
+      <c r="P2" s="0">
+        <v>68.680000000000007</v>
+      </c>
+      <c r="Q2" s="0">
+        <v>7.5199999999999996</v>
+      </c>
+      <c r="R2" s="0">
+        <v>20.850000000000001</v>
+      </c>
+      <c r="S2" s="0">
+        <v>3.3500000000000001</v>
+      </c>
+      <c r="T2" s="0">
+        <v>28.149999999999999</v>
+      </c>
+      <c r="U2" s="0">
+        <v>3.23</v>
+      </c>
+      <c r="V2" s="0">
+        <v>26.140000000000001</v>
+      </c>
+      <c r="W2" s="0">
+        <v>9.6899999999999995</v>
+      </c>
+      <c r="X2" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>10.08</v>
+      </c>
+      <c r="C3" s="0">
+        <v>7.1799999999999997</v>
+      </c>
+      <c r="D3" s="0">
+        <v>39.649999999999999</v>
+      </c>
+      <c r="E3" s="0">
+        <v>43.479999999999997</v>
+      </c>
+      <c r="F3" s="0">
+        <v>35.810000000000002</v>
+      </c>
+      <c r="G3" s="0">
+        <v>23.859999999999999</v>
+      </c>
+      <c r="H3" s="0">
+        <v>58.700000000000003</v>
+      </c>
+      <c r="I3" s="0">
+        <v>62.829999999999998</v>
+      </c>
+      <c r="J3" s="0">
+        <v>33.939999999999998</v>
+      </c>
+      <c r="K3" s="0">
+        <v>14.17</v>
+      </c>
+      <c r="L3" s="0">
+        <v>35.039999999999999</v>
+      </c>
+      <c r="M3" s="0">
+        <v>6.1299999999999999</v>
+      </c>
+      <c r="N3" s="0">
+        <v>80.659999999999997</v>
+      </c>
+      <c r="O3" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="P3" s="0">
+        <v>86.950000000000003</v>
+      </c>
+      <c r="Q3" s="0">
+        <v>15.35</v>
+      </c>
+      <c r="R3" s="0">
+        <v>25.379999999999999</v>
+      </c>
+      <c r="S3" s="0">
+        <v>5.6100000000000003</v>
+      </c>
+      <c r="T3" s="0">
+        <v>24.260000000000002</v>
+      </c>
+      <c r="U3" s="0">
+        <v>4</v>
+      </c>
+      <c r="V3" s="0">
+        <v>25.489999999999998</v>
+      </c>
+      <c r="W3" s="0">
+        <v>4.9500000000000002</v>
+      </c>
+      <c r="X3" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>45.18</v>
+      </c>
+      <c r="C4" s="0">
+        <v>48.07</v>
+      </c>
+      <c r="D4" s="0">
+        <v>48.890000000000001</v>
+      </c>
+      <c r="E4" s="0">
+        <v>83.019999999999996</v>
+      </c>
+      <c r="F4" s="0">
+        <v>30.829999999999998</v>
+      </c>
+      <c r="G4" s="0">
+        <v>26.829999999999998</v>
+      </c>
+      <c r="H4" s="0">
+        <v>24.309999999999999</v>
+      </c>
+      <c r="I4" s="0">
+        <v>14.15</v>
+      </c>
+      <c r="J4" s="0">
+        <v>31.699999999999999</v>
+      </c>
+      <c r="K4" s="0">
+        <v>23.260000000000002</v>
+      </c>
+      <c r="L4" s="0">
+        <v>78.170000000000002</v>
+      </c>
+      <c r="M4" s="0">
+        <v>10.18</v>
+      </c>
+      <c r="N4" s="0">
+        <v>53.350000000000001</v>
+      </c>
+      <c r="O4" s="0">
+        <v>6.1500000000000004</v>
+      </c>
+      <c r="P4" s="0">
+        <v>69.170000000000002</v>
+      </c>
+      <c r="Q4" s="0">
+        <v>6.2199999999999998</v>
+      </c>
+      <c r="R4" s="0">
+        <v>18.16</v>
+      </c>
+      <c r="S4" s="0">
+        <v>4.9100000000000001</v>
+      </c>
+      <c r="T4" s="0">
+        <v>29.07</v>
+      </c>
+      <c r="U4" s="0">
+        <v>4.0499999999999998</v>
+      </c>
+      <c r="V4" s="0">
+        <v>22.350000000000001</v>
+      </c>
+      <c r="W4" s="0">
+        <v>15.539999999999999</v>
+      </c>
+      <c r="X4" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>12.550000000000001</v>
+      </c>
+      <c r="C5" s="0">
+        <v>10.140000000000001</v>
+      </c>
+      <c r="D5" s="0">
+        <v>40.460000000000001</v>
+      </c>
+      <c r="E5" s="0">
+        <v>46.740000000000002</v>
+      </c>
+      <c r="F5" s="0">
+        <v>38.409999999999997</v>
+      </c>
+      <c r="G5" s="0">
+        <v>36.990000000000002</v>
+      </c>
+      <c r="H5" s="0">
+        <v>60.18</v>
+      </c>
+      <c r="I5" s="0">
+        <v>68.090000000000003</v>
+      </c>
+      <c r="J5" s="0">
+        <v>37.829999999999998</v>
+      </c>
+      <c r="K5" s="0">
+        <v>21.620000000000001</v>
+      </c>
+      <c r="L5" s="0">
+        <v>37.740000000000002</v>
+      </c>
+      <c r="M5" s="0">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="N5" s="0">
+        <v>93.290000000000006</v>
+      </c>
+      <c r="O5" s="0">
+        <v>13.69</v>
+      </c>
+      <c r="P5" s="0">
+        <v>93.260000000000005</v>
+      </c>
+      <c r="Q5" s="0">
+        <v>10.970000000000001</v>
+      </c>
+      <c r="R5" s="0">
+        <v>24.289999999999999</v>
+      </c>
+      <c r="S5" s="0">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="T5" s="0">
+        <v>23.350000000000001</v>
+      </c>
+      <c r="U5" s="0">
+        <v>5.2800000000000002</v>
+      </c>
+      <c r="V5" s="0">
+        <v>25.710000000000001</v>
+      </c>
+      <c r="W5" s="0">
+        <v>7.2800000000000002</v>
+      </c>
+      <c r="X5" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0">
+        <v>47.090000000000003</v>
+      </c>
+      <c r="C6" s="0">
+        <v>43</v>
+      </c>
+      <c r="D6" s="0">
+        <v>51.43</v>
+      </c>
+      <c r="E6" s="0">
+        <v>65.609999999999999</v>
+      </c>
+      <c r="F6" s="0">
+        <v>28.920000000000002</v>
+      </c>
+      <c r="G6" s="0">
+        <v>21.780000000000001</v>
+      </c>
+      <c r="H6" s="0">
+        <v>27.969999999999999</v>
+      </c>
+      <c r="I6" s="0">
+        <v>12.35</v>
+      </c>
+      <c r="J6" s="0">
+        <v>36.460000000000001</v>
+      </c>
+      <c r="K6" s="0">
+        <v>17.850000000000001</v>
+      </c>
+      <c r="L6" s="0">
+        <v>82.890000000000001</v>
+      </c>
+      <c r="M6" s="0">
+        <v>9.6400000000000006</v>
+      </c>
+      <c r="N6" s="0">
+        <v>52.950000000000003</v>
+      </c>
+      <c r="O6" s="0">
+        <v>5.9900000000000002</v>
+      </c>
+      <c r="P6" s="0">
+        <v>65.109999999999999</v>
+      </c>
+      <c r="Q6" s="0">
+        <v>9.0700000000000003</v>
+      </c>
+      <c r="R6" s="0">
+        <v>20.960000000000001</v>
+      </c>
+      <c r="S6" s="0">
+        <v>3.02</v>
+      </c>
+      <c r="T6" s="0">
+        <v>30.140000000000001</v>
+      </c>
+      <c r="U6" s="0">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="V6" s="0">
+        <v>20.699999999999999</v>
+      </c>
+      <c r="W6" s="0">
+        <v>12.26</v>
+      </c>
+      <c r="X6" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
         <v>6</v>
+      </c>
+      <c r="B7" s="0">
+        <v>10.24</v>
+      </c>
+      <c r="C7" s="0">
+        <v>7.1200000000000001</v>
+      </c>
+      <c r="D7" s="0">
+        <v>44.969999999999999</v>
+      </c>
+      <c r="E7" s="0">
+        <v>40.159999999999997</v>
+      </c>
+      <c r="F7" s="0">
+        <v>56.43</v>
+      </c>
+      <c r="G7" s="0">
+        <v>51.18</v>
+      </c>
+      <c r="H7" s="0">
+        <v>61.799999999999997</v>
+      </c>
+      <c r="I7" s="0">
+        <v>52.189999999999998</v>
+      </c>
+      <c r="J7" s="0">
+        <v>50.619999999999997</v>
+      </c>
+      <c r="K7" s="0">
+        <v>19.550000000000001</v>
+      </c>
+      <c r="L7" s="0">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="M7" s="0">
+        <v>8.0800000000000001</v>
+      </c>
+      <c r="N7" s="0">
+        <v>101.45999999999999</v>
+      </c>
+      <c r="O7" s="0">
+        <v>11.26</v>
+      </c>
+      <c r="P7" s="0">
+        <v>97.459999999999994</v>
+      </c>
+      <c r="Q7" s="0">
+        <v>13.619999999999999</v>
+      </c>
+      <c r="R7" s="0">
+        <v>25.41</v>
+      </c>
+      <c r="S7" s="0">
+        <v>4.3099999999999996</v>
+      </c>
+      <c r="T7" s="0">
+        <v>21.789999999999999</v>
+      </c>
+      <c r="U7" s="0">
+        <v>6.5700000000000003</v>
+      </c>
+      <c r="V7" s="0">
+        <v>24.579999999999998</v>
+      </c>
+      <c r="W7" s="0">
+        <v>9.5</v>
+      </c>
+      <c r="X7" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0">
+        <v>40.829999999999998</v>
+      </c>
+      <c r="C8" s="0">
+        <v>52.659999999999997</v>
+      </c>
+      <c r="D8" s="0">
+        <v>47.310000000000002</v>
+      </c>
+      <c r="E8" s="0">
+        <v>78.200000000000003</v>
+      </c>
+      <c r="F8" s="0">
+        <v>31.140000000000001</v>
+      </c>
+      <c r="G8" s="0">
+        <v>30.329999999999998</v>
+      </c>
+      <c r="H8" s="0">
+        <v>32.100000000000001</v>
+      </c>
+      <c r="I8" s="0">
+        <v>16.300000000000001</v>
+      </c>
+      <c r="J8" s="0">
+        <v>23.640000000000001</v>
+      </c>
+      <c r="K8" s="0">
+        <v>13.35</v>
+      </c>
+      <c r="L8" s="0">
+        <v>66.510000000000005</v>
+      </c>
+      <c r="M8" s="0">
+        <v>9.8399999999999999</v>
+      </c>
+      <c r="N8" s="0">
+        <v>51.700000000000003</v>
+      </c>
+      <c r="O8" s="0">
+        <v>5.6100000000000003</v>
+      </c>
+      <c r="P8" s="0">
+        <v>70.969999999999999</v>
+      </c>
+      <c r="Q8" s="0">
+        <v>6.7400000000000002</v>
+      </c>
+      <c r="R8" s="0">
+        <v>18.02</v>
+      </c>
+      <c r="S8" s="0">
+        <v>2.8300000000000001</v>
+      </c>
+      <c r="T8" s="0">
+        <v>31.300000000000001</v>
+      </c>
+      <c r="U8" s="0">
+        <v>3.8100000000000001</v>
+      </c>
+      <c r="V8" s="0">
+        <v>28.289999999999999</v>
+      </c>
+      <c r="W8" s="0">
+        <v>12.98</v>
+      </c>
+      <c r="X8" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>13.4</v>
+      </c>
+      <c r="C9" s="0">
+        <v>10.710000000000001</v>
+      </c>
+      <c r="D9" s="0">
+        <v>36.460000000000001</v>
+      </c>
+      <c r="E9" s="0">
+        <v>41.710000000000001</v>
+      </c>
+      <c r="F9" s="0">
+        <v>41.030000000000001</v>
+      </c>
+      <c r="G9" s="0">
+        <v>29.690000000000001</v>
+      </c>
+      <c r="H9" s="0">
+        <v>50.479999999999997</v>
+      </c>
+      <c r="I9" s="0">
+        <v>59.219999999999999</v>
+      </c>
+      <c r="J9" s="0">
+        <v>29.530000000000001</v>
+      </c>
+      <c r="K9" s="0">
+        <v>12.529999999999999</v>
+      </c>
+      <c r="L9" s="0">
+        <v>36.539999999999999</v>
+      </c>
+      <c r="M9" s="0">
+        <v>5.54</v>
+      </c>
+      <c r="N9" s="0">
+        <v>82.299999999999997</v>
+      </c>
+      <c r="O9" s="0">
+        <v>12.83</v>
+      </c>
+      <c r="P9" s="0">
+        <v>91.560000000000002</v>
+      </c>
+      <c r="Q9" s="0">
+        <v>14.81</v>
+      </c>
+      <c r="R9" s="0">
+        <v>24.84</v>
+      </c>
+      <c r="S9" s="0">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="T9" s="0">
+        <v>24.379999999999999</v>
+      </c>
+      <c r="U9" s="0">
+        <v>3.1499999999999999</v>
+      </c>
+      <c r="V9" s="0">
+        <v>26.030000000000001</v>
+      </c>
+      <c r="W9" s="0">
+        <v>7.1600000000000001</v>
+      </c>
+      <c r="X9" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>49.369999999999997</v>
+      </c>
+      <c r="C10" s="0">
+        <v>49.380000000000003</v>
+      </c>
+      <c r="D10" s="0">
+        <v>52.049999999999997</v>
+      </c>
+      <c r="E10" s="0">
+        <v>73.609999999999999</v>
+      </c>
+      <c r="F10" s="0">
+        <v>31.969999999999999</v>
+      </c>
+      <c r="G10" s="0">
+        <v>25.329999999999998</v>
+      </c>
+      <c r="H10" s="0">
+        <v>23.719999999999999</v>
+      </c>
+      <c r="I10" s="0">
+        <v>10.890000000000001</v>
+      </c>
+      <c r="J10" s="0">
+        <v>30.629999999999999</v>
+      </c>
+      <c r="K10" s="0">
+        <v>15.99</v>
+      </c>
+      <c r="L10" s="0">
+        <v>80.540000000000006</v>
+      </c>
+      <c r="M10" s="0">
+        <v>9.3499999999999996</v>
+      </c>
+      <c r="N10" s="0">
+        <v>53.719999999999999</v>
+      </c>
+      <c r="O10" s="0">
+        <v>5.4800000000000004</v>
+      </c>
+      <c r="P10" s="0">
+        <v>68.349999999999994</v>
+      </c>
+      <c r="Q10" s="0">
+        <v>5.4199999999999999</v>
+      </c>
+      <c r="R10" s="0">
+        <v>17.199999999999999</v>
+      </c>
+      <c r="S10" s="0">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="T10" s="0">
+        <v>31.140000000000001</v>
+      </c>
+      <c r="U10" s="0">
+        <v>3.6000000000000001</v>
+      </c>
+      <c r="V10" s="0">
+        <v>21.690000000000001</v>
+      </c>
+      <c r="W10" s="0">
+        <v>15.52</v>
+      </c>
+      <c r="X10" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>10.92</v>
+      </c>
+      <c r="C11" s="0">
+        <v>5.9900000000000002</v>
+      </c>
+      <c r="D11" s="0">
+        <v>38.25</v>
+      </c>
+      <c r="E11" s="0">
+        <v>40.950000000000003</v>
+      </c>
+      <c r="F11" s="0">
+        <v>36.560000000000002</v>
+      </c>
+      <c r="G11" s="0">
+        <v>31.629999999999999</v>
+      </c>
+      <c r="H11" s="0">
+        <v>60.009999999999998</v>
+      </c>
+      <c r="I11" s="0">
+        <v>58.759999999999998</v>
+      </c>
+      <c r="J11" s="0">
+        <v>41.799999999999997</v>
+      </c>
+      <c r="K11" s="0">
+        <v>18.199999999999999</v>
+      </c>
+      <c r="L11" s="0">
+        <v>38.439999999999998</v>
+      </c>
+      <c r="M11" s="0">
+        <v>7.0199999999999996</v>
+      </c>
+      <c r="N11" s="0">
+        <v>95.650000000000006</v>
+      </c>
+      <c r="O11" s="0">
+        <v>12.390000000000001</v>
+      </c>
+      <c r="P11" s="0">
+        <v>95.280000000000001</v>
+      </c>
+      <c r="Q11" s="0">
+        <v>13.130000000000001</v>
+      </c>
+      <c r="R11" s="0">
+        <v>24.760000000000002</v>
+      </c>
+      <c r="S11" s="0">
+        <v>5.8099999999999996</v>
+      </c>
+      <c r="T11" s="0">
+        <v>20.18</v>
+      </c>
+      <c r="U11" s="0">
+        <v>5.5800000000000001</v>
+      </c>
+      <c r="V11" s="0">
+        <v>22.510000000000002</v>
+      </c>
+      <c r="W11" s="0">
+        <v>6.0700000000000003</v>
+      </c>
+      <c r="X11" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0">
+        <v>56.890000000000001</v>
+      </c>
+      <c r="C12" s="0">
+        <v>52.420000000000002</v>
+      </c>
+      <c r="D12" s="0">
+        <v>64.719999999999999</v>
+      </c>
+      <c r="E12" s="0">
+        <v>79.579999999999998</v>
+      </c>
+      <c r="F12" s="0">
+        <v>33.890000000000001</v>
+      </c>
+      <c r="G12" s="0">
+        <v>26.98</v>
+      </c>
+      <c r="H12" s="0">
+        <v>31.829999999999998</v>
+      </c>
+      <c r="I12" s="0">
+        <v>11.75</v>
+      </c>
+      <c r="J12" s="0">
+        <v>27.98</v>
+      </c>
+      <c r="K12" s="0">
+        <v>12.35</v>
+      </c>
+      <c r="L12" s="0">
+        <v>88.109999999999999</v>
+      </c>
+      <c r="M12" s="0">
+        <v>8.2100000000000009</v>
+      </c>
+      <c r="N12" s="0">
+        <v>53.340000000000003</v>
+      </c>
+      <c r="O12" s="0">
+        <v>6.5</v>
+      </c>
+      <c r="P12" s="0">
+        <v>68.359999999999999</v>
+      </c>
+      <c r="Q12" s="0">
+        <v>7.8200000000000003</v>
+      </c>
+      <c r="R12" s="0">
+        <v>18.760000000000002</v>
+      </c>
+      <c r="S12" s="0">
+        <v>4.3300000000000001</v>
+      </c>
+      <c r="T12" s="0">
+        <v>29.239999999999998</v>
+      </c>
+      <c r="U12" s="0">
+        <v>4.3799999999999999</v>
+      </c>
+      <c r="V12" s="0">
+        <v>17.77</v>
+      </c>
+      <c r="W12" s="0">
+        <v>12.91</v>
+      </c>
+      <c r="X12" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0">
+        <v>9.9600000000000009</v>
+      </c>
+      <c r="C13" s="0">
+        <v>6.8700000000000001</v>
+      </c>
+      <c r="D13" s="0">
+        <v>45.670000000000002</v>
+      </c>
+      <c r="E13" s="0">
+        <v>42.630000000000003</v>
+      </c>
+      <c r="F13" s="0">
+        <v>45.100000000000001</v>
+      </c>
+      <c r="G13" s="0">
+        <v>33.719999999999999</v>
+      </c>
+      <c r="H13" s="0">
+        <v>55.82</v>
+      </c>
+      <c r="I13" s="0">
+        <v>57.799999999999997</v>
+      </c>
+      <c r="J13" s="0">
+        <v>59.759999999999998</v>
+      </c>
+      <c r="K13" s="0">
+        <v>22.280000000000001</v>
+      </c>
+      <c r="L13" s="0">
+        <v>42.329999999999998</v>
+      </c>
+      <c r="M13" s="0">
+        <v>9.3399999999999999</v>
+      </c>
+      <c r="N13" s="0">
+        <v>108.52</v>
+      </c>
+      <c r="O13" s="0">
+        <v>13.279999999999999</v>
+      </c>
+      <c r="P13" s="0">
+        <v>101.37</v>
+      </c>
+      <c r="Q13" s="0">
+        <v>11.24</v>
+      </c>
+      <c r="R13" s="0">
+        <v>25.559999999999999</v>
+      </c>
+      <c r="S13" s="0">
+        <v>2.6800000000000002</v>
+      </c>
+      <c r="T13" s="0">
+        <v>23.890000000000001</v>
+      </c>
+      <c r="U13" s="0">
+        <v>3.8900000000000001</v>
+      </c>
+      <c r="V13" s="0">
+        <v>25.539999999999999</v>
+      </c>
+      <c r="W13" s="0">
+        <v>8.6099999999999994</v>
+      </c>
+      <c r="X13" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="0">
+        <v>12.029999999999999</v>
+      </c>
+      <c r="C14" s="0">
+        <v>3.96</v>
+      </c>
+      <c r="D14" s="0">
+        <v>10.84</v>
+      </c>
+      <c r="E14" s="0">
+        <v>5.9100000000000001</v>
+      </c>
+      <c r="F14" s="0">
+        <v>29.620000000000001</v>
+      </c>
+      <c r="G14" s="0">
+        <v>17.5</v>
+      </c>
+      <c r="H14" s="0">
+        <v>24.52</v>
+      </c>
+      <c r="I14" s="0">
+        <v>13.68</v>
+      </c>
+      <c r="J14" s="0">
+        <v>12.130000000000001</v>
+      </c>
+      <c r="K14" s="0">
+        <v>2.3100000000000001</v>
+      </c>
+      <c r="L14" s="0">
+        <v>26.300000000000001</v>
+      </c>
+      <c r="M14" s="0">
+        <v>3.1299999999999999</v>
+      </c>
+      <c r="N14" s="0">
+        <v>48.450000000000003</v>
+      </c>
+      <c r="O14" s="0">
+        <v>5.21</v>
+      </c>
+      <c r="P14" s="0">
+        <v>68.290000000000006</v>
+      </c>
+      <c r="Q14" s="0">
+        <v>5.8300000000000001</v>
+      </c>
+      <c r="R14" s="0">
+        <v>18.789999999999999</v>
+      </c>
+      <c r="S14" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="T14" s="0">
+        <v>26.699999999999999</v>
+      </c>
+      <c r="U14" s="0">
+        <v>2.04</v>
+      </c>
+      <c r="V14" s="0">
+        <v>24.07</v>
+      </c>
+      <c r="W14" s="0">
+        <v>3.3900000000000001</v>
+      </c>
+      <c r="X14" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" customWidth="true"/>
+    <col min="2" max="2" width="17.5703125" customWidth="true"/>
+    <col min="3" max="3" width="14.85546875" customWidth="true"/>
+    <col min="4" max="4" width="19.140625" customWidth="true"/>
+    <col min="5" max="5" width="16.42578125" customWidth="true"/>
+    <col min="6" max="6" width="15.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13" customWidth="true"/>
+    <col min="8" max="8" width="15.85546875" customWidth="true"/>
+    <col min="9" max="9" width="13.140625" customWidth="true"/>
+    <col min="10" max="10" width="17" customWidth="true"/>
+    <col min="11" max="11" width="14.28515625" customWidth="true"/>
+    <col min="12" max="12" width="16.140625" customWidth="true"/>
+    <col min="13" max="13" width="13.42578125" customWidth="true"/>
+    <col min="14" max="14" width="17.28515625" customWidth="true"/>
+    <col min="15" max="15" width="14.5703125" customWidth="true"/>
+    <col min="16" max="16" width="19.85546875" customWidth="true"/>
+    <col min="17" max="17" width="17.140625" customWidth="true"/>
+    <col min="18" max="18" width="16.7109375" customWidth="true"/>
+    <col min="19" max="19" width="14" customWidth="true"/>
+    <col min="20" max="20" width="16.7109375" customWidth="true"/>
+    <col min="21" max="21" width="14" customWidth="true"/>
+    <col min="22" max="22" width="17.140625" customWidth="true"/>
+    <col min="23" max="23" width="14.42578125" customWidth="true"/>
+    <col min="24" max="24" width="13.7109375" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="T1" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>33.020000000000003</v>
+      </c>
+      <c r="C2" s="0">
+        <v>53.109999999999999</v>
+      </c>
+      <c r="D2" s="0">
+        <v>41.130000000000003</v>
+      </c>
+      <c r="E2" s="0">
+        <v>83.709999999999994</v>
+      </c>
+      <c r="F2" s="0">
+        <v>4.0800000000000001</v>
+      </c>
+      <c r="G2" s="0">
+        <v>18.920000000000002</v>
+      </c>
+      <c r="H2" s="0">
+        <v>3.6299999999999999</v>
+      </c>
+      <c r="I2" s="0">
+        <v>13.08</v>
+      </c>
+      <c r="J2" s="0">
+        <v>10.23</v>
+      </c>
+      <c r="K2" s="0">
+        <v>6.75</v>
+      </c>
+      <c r="L2" s="0">
+        <v>36.079999999999998</v>
+      </c>
+      <c r="M2" s="0">
+        <v>9.5800000000000001</v>
+      </c>
+      <c r="N2" s="0">
+        <v>3.5600000000000001</v>
+      </c>
+      <c r="O2" s="0">
+        <v>3.1499999999999999</v>
+      </c>
+      <c r="P2" s="0">
+        <v>0.38</v>
+      </c>
+      <c r="Q2" s="0">
+        <v>4.8300000000000001</v>
+      </c>
+      <c r="R2" s="0">
+        <v>1.49</v>
+      </c>
+      <c r="S2" s="0">
+        <v>2.52</v>
+      </c>
+      <c r="T2" s="0">
+        <v>1.45</v>
+      </c>
+      <c r="U2" s="0">
+        <v>3.4300000000000002</v>
+      </c>
+      <c r="V2" s="0">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="W2" s="0">
+        <v>8.9700000000000006</v>
+      </c>
+      <c r="X2" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>-2.4399999999999999</v>
+      </c>
+      <c r="C3" s="0">
+        <v>8.1500000000000004</v>
+      </c>
+      <c r="D3" s="0">
+        <v>27.829999999999998</v>
+      </c>
+      <c r="E3" s="0">
+        <v>40.469999999999999</v>
+      </c>
+      <c r="F3" s="0">
+        <v>6.1900000000000004</v>
+      </c>
+      <c r="G3" s="0">
+        <v>21.43</v>
+      </c>
+      <c r="H3" s="0">
+        <v>34.18</v>
+      </c>
+      <c r="I3" s="0">
+        <v>52.140000000000001</v>
+      </c>
+      <c r="J3" s="0">
+        <v>22.010000000000002</v>
+      </c>
+      <c r="K3" s="0">
+        <v>13.300000000000001</v>
+      </c>
+      <c r="L3" s="0">
+        <v>8.2400000000000002</v>
+      </c>
+      <c r="M3" s="0">
+        <v>4.0599999999999996</v>
+      </c>
+      <c r="N3" s="0">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="O3" s="0">
+        <v>14.449999999999999</v>
+      </c>
+      <c r="P3" s="0">
+        <v>18.66</v>
+      </c>
+      <c r="Q3" s="0">
+        <v>11.800000000000001</v>
+      </c>
+      <c r="R3" s="0">
+        <v>6.0199999999999996</v>
+      </c>
+      <c r="S3" s="0">
+        <v>4.7400000000000002</v>
+      </c>
+      <c r="T3" s="0">
+        <v>-2.4399999999999999</v>
+      </c>
+      <c r="U3" s="0">
+        <v>3.4100000000000001</v>
+      </c>
+      <c r="V3" s="0">
+        <v>1.4099999999999999</v>
+      </c>
+      <c r="W3" s="0">
+        <v>3.2999999999999998</v>
+      </c>
+      <c r="X3" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>33.149999999999999</v>
+      </c>
+      <c r="C4" s="0">
+        <v>49.390000000000001</v>
+      </c>
+      <c r="D4" s="0">
+        <v>38.039999999999999</v>
+      </c>
+      <c r="E4" s="0">
+        <v>81.319999999999993</v>
+      </c>
+      <c r="F4" s="0">
+        <v>1.21</v>
+      </c>
+      <c r="G4" s="0">
+        <v>20.420000000000002</v>
+      </c>
+      <c r="H4" s="0">
+        <v>-0.20000000000000001</v>
+      </c>
+      <c r="I4" s="0">
+        <v>14.460000000000001</v>
+      </c>
+      <c r="J4" s="0">
+        <v>19.57</v>
+      </c>
+      <c r="K4" s="0">
+        <v>21.829999999999998</v>
+      </c>
+      <c r="L4" s="0">
+        <v>51.869999999999997</v>
+      </c>
+      <c r="M4" s="0">
+        <v>9.1300000000000008</v>
+      </c>
+      <c r="N4" s="0">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="O4" s="0">
+        <v>3.6699999999999999</v>
+      </c>
+      <c r="P4" s="0">
+        <v>0.88</v>
+      </c>
+      <c r="Q4" s="0">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="R4" s="0">
+        <v>-0.63</v>
+      </c>
+      <c r="S4" s="0">
+        <v>2.5</v>
+      </c>
+      <c r="T4" s="0">
+        <v>2.3700000000000001</v>
+      </c>
+      <c r="U4" s="0">
+        <v>4.9900000000000002</v>
+      </c>
+      <c r="V4" s="0">
+        <v>-1.73</v>
+      </c>
+      <c r="W4" s="0">
+        <v>14.48</v>
+      </c>
+      <c r="X4" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.53000000000000003</v>
+      </c>
+      <c r="C5" s="0">
+        <v>7.8200000000000003</v>
+      </c>
+      <c r="D5" s="0">
+        <v>29.620000000000001</v>
+      </c>
+      <c r="E5" s="0">
+        <v>42.560000000000002</v>
+      </c>
+      <c r="F5" s="0">
+        <v>8.7899999999999991</v>
+      </c>
+      <c r="G5" s="0">
+        <v>30.030000000000001</v>
+      </c>
+      <c r="H5" s="0">
+        <v>35.659999999999997</v>
+      </c>
+      <c r="I5" s="0">
+        <v>56.939999999999998</v>
+      </c>
+      <c r="J5" s="0">
+        <v>25.699999999999999</v>
+      </c>
+      <c r="K5" s="0">
+        <v>20.960000000000001</v>
+      </c>
+      <c r="L5" s="0">
+        <v>11.43</v>
+      </c>
+      <c r="M5" s="0">
+        <v>5.0899999999999999</v>
+      </c>
+      <c r="N5" s="0">
+        <v>44.829999999999998</v>
+      </c>
+      <c r="O5" s="0">
+        <v>13.56</v>
+      </c>
+      <c r="P5" s="0">
+        <v>24.960000000000001</v>
+      </c>
+      <c r="Q5" s="0">
+        <v>7.9100000000000001</v>
+      </c>
+      <c r="R5" s="0">
+        <v>5.5</v>
+      </c>
+      <c r="S5" s="0">
+        <v>3.46</v>
+      </c>
+      <c r="T5" s="0">
+        <v>-3.3500000000000001</v>
+      </c>
+      <c r="U5" s="0">
+        <v>4.2599999999999998</v>
+      </c>
+      <c r="V5" s="0">
+        <v>1.6399999999999999</v>
+      </c>
+      <c r="W5" s="0">
+        <v>5.3799999999999999</v>
+      </c>
+      <c r="X5" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0">
+        <v>34.579999999999998</v>
+      </c>
+      <c r="C6" s="0">
+        <v>45.420000000000002</v>
+      </c>
+      <c r="D6" s="0">
+        <v>39.609999999999999</v>
+      </c>
+      <c r="E6" s="0">
+        <v>63.490000000000002</v>
+      </c>
+      <c r="F6" s="0">
+        <v>-0.69999999999999996</v>
+      </c>
+      <c r="G6" s="0">
+        <v>12.31</v>
+      </c>
+      <c r="H6" s="0">
+        <v>3.4500000000000002</v>
+      </c>
+      <c r="I6" s="0">
+        <v>14.859999999999999</v>
+      </c>
+      <c r="J6" s="0">
+        <v>24.530000000000001</v>
+      </c>
+      <c r="K6" s="0">
+        <v>15.67</v>
+      </c>
+      <c r="L6" s="0">
+        <v>56.090000000000003</v>
+      </c>
+      <c r="M6" s="0">
+        <v>7.4900000000000002</v>
+      </c>
+      <c r="N6" s="0">
+        <v>4.4900000000000002</v>
+      </c>
+      <c r="O6" s="0">
+        <v>3.1499999999999999</v>
+      </c>
+      <c r="P6" s="0">
+        <v>-3.1800000000000002</v>
+      </c>
+      <c r="Q6" s="0">
+        <v>11.050000000000001</v>
+      </c>
+      <c r="R6" s="0">
+        <v>1.6000000000000001</v>
+      </c>
+      <c r="S6" s="0">
+        <v>5.5499999999999998</v>
+      </c>
+      <c r="T6" s="0">
+        <v>3.4399999999999999</v>
+      </c>
+      <c r="U6" s="0">
+        <v>5.3799999999999999</v>
+      </c>
+      <c r="V6" s="0">
+        <v>-3.3799999999999999</v>
+      </c>
+      <c r="W6" s="0">
+        <v>12.029999999999999</v>
+      </c>
+      <c r="X6" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0">
+        <v>-2.2799999999999998</v>
+      </c>
+      <c r="C7" s="0">
+        <v>7.8399999999999999</v>
+      </c>
+      <c r="D7" s="0">
+        <v>33.149999999999999</v>
+      </c>
+      <c r="E7" s="0">
+        <v>34.969999999999999</v>
+      </c>
+      <c r="F7" s="0">
+        <v>26.809999999999999</v>
+      </c>
+      <c r="G7" s="0">
+        <v>50.18</v>
+      </c>
+      <c r="H7" s="0">
+        <v>37.280000000000001</v>
+      </c>
+      <c r="I7" s="0">
+        <v>42.219999999999999</v>
+      </c>
+      <c r="J7" s="0">
+        <v>38.689999999999998</v>
+      </c>
+      <c r="K7" s="0">
+        <v>19.609999999999999</v>
+      </c>
+      <c r="L7" s="0">
+        <v>13.4</v>
+      </c>
+      <c r="M7" s="0">
+        <v>6.2000000000000002</v>
+      </c>
+      <c r="N7" s="0">
+        <v>53</v>
+      </c>
+      <c r="O7" s="0">
+        <v>10.460000000000001</v>
+      </c>
+      <c r="P7" s="0">
+        <v>29.170000000000002</v>
+      </c>
+      <c r="Q7" s="0">
+        <v>12.65</v>
+      </c>
+      <c r="R7" s="0">
+        <v>6.0499999999999998</v>
+      </c>
+      <c r="S7" s="0">
+        <v>2.6499999999999999</v>
+      </c>
+      <c r="T7" s="0">
+        <v>-4.9100000000000001</v>
+      </c>
+      <c r="U7" s="0">
+        <v>6.5199999999999996</v>
+      </c>
+      <c r="V7" s="0">
+        <v>0.51000000000000001</v>
+      </c>
+      <c r="W7" s="0">
+        <v>8.2400000000000002</v>
+      </c>
+      <c r="X7" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0">
+        <v>28.809999999999999</v>
+      </c>
+      <c r="C8" s="0">
+        <v>53.130000000000003</v>
+      </c>
+      <c r="D8" s="0">
+        <v>36.460000000000001</v>
+      </c>
+      <c r="E8" s="0">
+        <v>76.219999999999999</v>
+      </c>
+      <c r="F8" s="0">
+        <v>1.52</v>
+      </c>
+      <c r="G8" s="0">
+        <v>20.530000000000001</v>
+      </c>
+      <c r="H8" s="0">
+        <v>7.5899999999999999</v>
+      </c>
+      <c r="I8" s="0">
+        <v>8.6899999999999995</v>
+      </c>
+      <c r="J8" s="0">
+        <v>11.51</v>
+      </c>
+      <c r="K8" s="0">
+        <v>11.609999999999999</v>
+      </c>
+      <c r="L8" s="0">
+        <v>40.210000000000001</v>
+      </c>
+      <c r="M8" s="0">
+        <v>7.0300000000000002</v>
+      </c>
+      <c r="N8" s="0">
+        <v>3.25</v>
+      </c>
+      <c r="O8" s="0">
+        <v>2.6499999999999999</v>
+      </c>
+      <c r="P8" s="0">
+        <v>2.6699999999999999</v>
+      </c>
+      <c r="Q8" s="0">
+        <v>3.0099999999999998</v>
+      </c>
+      <c r="R8" s="0">
+        <v>-0.77000000000000002</v>
+      </c>
+      <c r="S8" s="0">
+        <v>2.8799999999999999</v>
+      </c>
+      <c r="T8" s="0">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="U8" s="0">
+        <v>4.8200000000000003</v>
+      </c>
+      <c r="V8" s="0">
+        <v>4.2199999999999998</v>
+      </c>
+      <c r="W8" s="0">
+        <v>12.85</v>
+      </c>
+      <c r="X8" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>1.3700000000000001</v>
+      </c>
+      <c r="C9" s="0">
+        <v>9.4299999999999997</v>
+      </c>
+      <c r="D9" s="0">
+        <v>25.620000000000001</v>
+      </c>
+      <c r="E9" s="0">
+        <v>37.609999999999999</v>
+      </c>
+      <c r="F9" s="0">
+        <v>11.41</v>
+      </c>
+      <c r="G9" s="0">
+        <v>27.370000000000001</v>
+      </c>
+      <c r="H9" s="0">
+        <v>25.969999999999999</v>
+      </c>
+      <c r="I9" s="0">
+        <v>49.18</v>
+      </c>
+      <c r="J9" s="0">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="K9" s="0">
+        <v>11.66</v>
+      </c>
+      <c r="L9" s="0">
+        <v>10.24</v>
+      </c>
+      <c r="M9" s="0">
+        <v>4.29</v>
+      </c>
+      <c r="N9" s="0">
+        <v>33.840000000000003</v>
+      </c>
+      <c r="O9" s="0">
+        <v>12.140000000000001</v>
+      </c>
+      <c r="P9" s="0">
+        <v>23.27</v>
+      </c>
+      <c r="Q9" s="0">
+        <v>12.15</v>
+      </c>
+      <c r="R9" s="0">
+        <v>6.04</v>
+      </c>
+      <c r="S9" s="0">
+        <v>3.7400000000000002</v>
+      </c>
+      <c r="T9" s="0">
+        <v>-2.3300000000000001</v>
+      </c>
+      <c r="U9" s="0">
+        <v>3.48</v>
+      </c>
+      <c r="V9" s="0">
+        <v>1.96</v>
+      </c>
+      <c r="W9" s="0">
+        <v>6.2300000000000004</v>
+      </c>
+      <c r="X9" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>37.340000000000003</v>
+      </c>
+      <c r="C10" s="0">
+        <v>50.979999999999997</v>
+      </c>
+      <c r="D10" s="0">
+        <v>41.210000000000001</v>
+      </c>
+      <c r="E10" s="0">
+        <v>71.140000000000001</v>
+      </c>
+      <c r="F10" s="0">
+        <v>2.3500000000000001</v>
+      </c>
+      <c r="G10" s="0">
+        <v>15.19</v>
+      </c>
+      <c r="H10" s="0">
+        <v>-0.80000000000000004</v>
+      </c>
+      <c r="I10" s="0">
+        <v>13.01</v>
+      </c>
+      <c r="J10" s="0">
+        <v>18.5</v>
+      </c>
+      <c r="K10" s="0">
+        <v>14.029999999999999</v>
+      </c>
+      <c r="L10" s="0">
+        <v>54.229999999999997</v>
+      </c>
+      <c r="M10" s="0">
+        <v>7.5999999999999996</v>
+      </c>
+      <c r="N10" s="0">
+        <v>5.2599999999999998</v>
+      </c>
+      <c r="O10" s="0">
+        <v>1.6200000000000001</v>
+      </c>
+      <c r="P10" s="0">
+        <v>0.050000000000000003</v>
+      </c>
+      <c r="Q10" s="0">
+        <v>5.7000000000000002</v>
+      </c>
+      <c r="R10" s="0">
+        <v>-1.5900000000000001</v>
+      </c>
+      <c r="S10" s="0">
+        <v>2.29</v>
+      </c>
+      <c r="T10" s="0">
+        <v>4.4400000000000004</v>
+      </c>
+      <c r="U10" s="0">
+        <v>4.4100000000000001</v>
+      </c>
+      <c r="V10" s="0">
+        <v>-2.3799999999999999</v>
+      </c>
+      <c r="W10" s="0">
+        <v>14.31</v>
+      </c>
+      <c r="X10" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="C11" s="0">
+        <v>5.5199999999999996</v>
+      </c>
+      <c r="D11" s="0">
+        <v>27.41</v>
+      </c>
+      <c r="E11" s="0">
+        <v>36.409999999999997</v>
+      </c>
+      <c r="F11" s="0">
+        <v>6.9400000000000004</v>
+      </c>
+      <c r="G11" s="0">
+        <v>29.359999999999999</v>
+      </c>
+      <c r="H11" s="0">
+        <v>35.5</v>
+      </c>
+      <c r="I11" s="0">
+        <v>47.990000000000002</v>
+      </c>
+      <c r="J11" s="0">
+        <v>29.670000000000002</v>
+      </c>
+      <c r="K11" s="0">
+        <v>18.640000000000001</v>
+      </c>
+      <c r="L11" s="0">
+        <v>12.140000000000001</v>
+      </c>
+      <c r="M11" s="0">
+        <v>6.9800000000000004</v>
+      </c>
+      <c r="N11" s="0">
+        <v>47.189999999999998</v>
+      </c>
+      <c r="O11" s="0">
+        <v>11.199999999999999</v>
+      </c>
+      <c r="P11" s="0">
+        <v>26.98</v>
+      </c>
+      <c r="Q11" s="0">
+        <v>10.98</v>
+      </c>
+      <c r="R11" s="0">
+        <v>5.96</v>
+      </c>
+      <c r="S11" s="0">
+        <v>4.5700000000000003</v>
+      </c>
+      <c r="T11" s="0">
+        <v>-6.5199999999999996</v>
+      </c>
+      <c r="U11" s="0">
+        <v>5.7300000000000004</v>
+      </c>
+      <c r="V11" s="0">
+        <v>-1.5600000000000001</v>
+      </c>
+      <c r="W11" s="0">
+        <v>5.6100000000000003</v>
+      </c>
+      <c r="X11" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0">
+        <v>44.380000000000003</v>
+      </c>
+      <c r="C12" s="0">
+        <v>54.880000000000003</v>
+      </c>
+      <c r="D12" s="0">
+        <v>52.890000000000001</v>
+      </c>
+      <c r="E12" s="0">
+        <v>77.819999999999993</v>
+      </c>
+      <c r="F12" s="0">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="G12" s="0">
+        <v>16.629999999999999</v>
+      </c>
+      <c r="H12" s="0">
+        <v>7.3200000000000003</v>
+      </c>
+      <c r="I12" s="0">
+        <v>6.5999999999999996</v>
+      </c>
+      <c r="J12" s="0">
+        <v>16.050000000000001</v>
+      </c>
+      <c r="K12" s="0">
+        <v>10.48</v>
+      </c>
+      <c r="L12" s="0">
+        <v>61.310000000000002</v>
+      </c>
+      <c r="M12" s="0">
+        <v>6.3600000000000003</v>
+      </c>
+      <c r="N12" s="0">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="O12" s="0">
+        <v>3.0899999999999999</v>
+      </c>
+      <c r="P12" s="0">
+        <v>0.059999999999999998</v>
+      </c>
+      <c r="Q12" s="0">
+        <v>5.0099999999999998</v>
+      </c>
+      <c r="R12" s="0">
+        <v>-0.59999999999999998</v>
+      </c>
+      <c r="S12" s="0">
+        <v>3.5800000000000001</v>
+      </c>
+      <c r="T12" s="0">
+        <v>2.54</v>
+      </c>
+      <c r="U12" s="0">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="V12" s="0">
+        <v>-6.2999999999999998</v>
+      </c>
+      <c r="W12" s="0">
+        <v>11.35</v>
+      </c>
+      <c r="X12" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0">
+        <v>-2.5499999999999998</v>
+      </c>
+      <c r="C13" s="0">
+        <v>7.9000000000000004</v>
+      </c>
+      <c r="D13" s="0">
+        <v>33.850000000000001</v>
+      </c>
+      <c r="E13" s="0">
+        <v>39.130000000000003</v>
+      </c>
+      <c r="F13" s="0">
+        <v>15.48</v>
+      </c>
+      <c r="G13" s="0">
+        <v>31.460000000000001</v>
+      </c>
+      <c r="H13" s="0">
+        <v>31.309999999999999</v>
+      </c>
+      <c r="I13" s="0">
+        <v>48.030000000000001</v>
+      </c>
+      <c r="J13" s="0">
+        <v>47.829999999999998</v>
+      </c>
+      <c r="K13" s="0">
+        <v>22.449999999999999</v>
+      </c>
+      <c r="L13" s="0">
+        <v>15.529999999999999</v>
+      </c>
+      <c r="M13" s="0">
+        <v>8.6400000000000006</v>
+      </c>
+      <c r="N13" s="0">
+        <v>60.060000000000002</v>
+      </c>
+      <c r="O13" s="0">
+        <v>13.65</v>
+      </c>
+      <c r="P13" s="0">
+        <v>33.079999999999998</v>
+      </c>
+      <c r="Q13" s="0">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="R13" s="0">
+        <v>6.2000000000000002</v>
+      </c>
+      <c r="S13" s="0">
+        <v>4.3799999999999999</v>
+      </c>
+      <c r="T13" s="0">
+        <v>-2.8199999999999998</v>
+      </c>
+      <c r="U13" s="0">
+        <v>3.5600000000000001</v>
+      </c>
+      <c r="V13" s="0">
+        <v>1.47</v>
+      </c>
+      <c r="W13" s="0">
+        <v>7.0300000000000002</v>
+      </c>
+      <c r="X13" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="0">
+        <v>0</v>
+      </c>
+      <c r="C14" s="0">
+        <v>0</v>
+      </c>
+      <c r="D14" s="0">
+        <v>0</v>
+      </c>
+      <c r="E14" s="0">
+        <v>0</v>
+      </c>
+      <c r="F14" s="0">
+        <v>0</v>
+      </c>
+      <c r="G14" s="0">
+        <v>0</v>
+      </c>
+      <c r="H14" s="0">
+        <v>0</v>
+      </c>
+      <c r="I14" s="0">
+        <v>0</v>
+      </c>
+      <c r="J14" s="0">
+        <v>0</v>
+      </c>
+      <c r="K14" s="0">
+        <v>0</v>
+      </c>
+      <c r="L14" s="0">
+        <v>0</v>
+      </c>
+      <c r="M14" s="0">
+        <v>0</v>
+      </c>
+      <c r="N14" s="0">
+        <v>0</v>
+      </c>
+      <c r="O14" s="0">
+        <v>0</v>
+      </c>
+      <c r="P14" s="0">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="0">
+        <v>0</v>
+      </c>
+      <c r="R14" s="0">
+        <v>0</v>
+      </c>
+      <c r="S14" s="0">
+        <v>0</v>
+      </c>
+      <c r="T14" s="0">
+        <v>0</v>
+      </c>
+      <c r="U14" s="0">
+        <v>0</v>
+      </c>
+      <c r="V14" s="0">
+        <v>0</v>
+      </c>
+      <c r="W14" s="0">
+        <v>0</v>
+      </c>
+      <c r="X14" s="0">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>